<commit_message>
Added a second test cell
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Publication" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="186">
   <si>
     <t xml:space="preserve">Item name</t>
   </si>
@@ -541,6 +541,9 @@
   </si>
   <si>
     <t xml:space="preserve">Microhomolgy of GA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEST</t>
   </si>
   <si>
     <t xml:space="preserve">n/a</t>
@@ -681,67 +684,67 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2845,7 +2848,9 @@
       <c r="D12" s="15" t="n">
         <v>126965660</v>
       </c>
-      <c r="E12" s="15"/>
+      <c r="E12" s="15" t="s">
+        <v>173</v>
+      </c>
       <c r="F12" s="11"/>
       <c r="G12" s="5"/>
     </row>
@@ -2934,10 +2939,10 @@
         <v>672515</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="18" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2974,10 +2979,10 @@
         <v>609000</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="20" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3014,10 +3019,10 @@
         <v>474998</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="22" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3054,10 +3059,10 @@
         <v>250000</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="24" s="4" customFormat="true" ht="73.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3080,7 +3085,7 @@
         <v>160</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="25" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3120,7 +3125,7 @@
         <v>160</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="27" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3143,7 +3148,7 @@
         <v>160</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="28" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3166,7 +3171,7 @@
         <v>160</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="29" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3189,7 +3194,7 @@
         <v>160</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="30" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3212,7 +3217,7 @@
         <v>160</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="31" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
ADLD_dup_30 track wasn't in Excel
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Publication" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="185">
   <si>
     <t xml:space="preserve">Item name</t>
   </si>
@@ -3322,10 +3322,18 @@
       <c r="G36" s="5"/>
     </row>
     <row r="37" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5"/>
-      <c r="B37" s="5"/>
-      <c r="C37" s="16"/>
-      <c r="D37" s="16"/>
+      <c r="A37" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="C37" s="16" t="n">
+        <v>126676469</v>
+      </c>
+      <c r="D37" s="16" t="n">
+        <v>126897351</v>
+      </c>
       <c r="E37" s="15"/>
       <c r="F37" s="11"/>
       <c r="G37" s="5"/>

</xml_diff>

<commit_message>
test - two cells with spaces between patients sx
testing ADLD_dup_1 and ADLD_dup_29
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\Krizchelle\ADLD Patient Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B2053C6-7829-4CC1-8FDE-AB235058FBE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9672A1B2-89B3-4306-8B8A-1008DA86F5EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Molecular" sheetId="4" r:id="rId1"/>
@@ -97,9 +97,6 @@
     <t>Canada</t>
   </si>
   <si>
-    <t>Bladder/bowel disturbances, lower limb weakness, orthostatic hypotension, impotence, decreased sweating, temperature dysregulation, ataxia, MRI showing leukodystrophy, lower limb hyperreflexia with occasional upper limb involvement</t>
-  </si>
-  <si>
     <t>10.1002/humu.22348, 10.1007/s10048-010-0269-y</t>
   </si>
   <si>
@@ -616,9 +613,6 @@
     <t>Negative family history, + autonomic disturbance, + pyramidal signs, + Ataxia, Cognitive impairment +MMSE23, MRI findings with MCP lesion</t>
   </si>
   <si>
-    <t>Three family members - symptoms listed in the Master Excel. Too lengthy place here at the current status of the website</t>
-  </si>
-  <si>
     <t>Pedigree I - Patient I</t>
   </si>
   <si>
@@ -689,6 +683,18 @@
   </si>
   <si>
     <t>Pedigree III - Patient 4</t>
+  </si>
+  <si>
+    <t>Symptoms in this family usually presented early in their 5th decade of life and consisted of bladder and/or bowel disturbances, lower limb weakness, orthostatic hypotension, and/or impotence. Disease progresses slowly and sometimes seems to remit. 
+II-2 and II-4 were said to be “crawling on the floor” in their 50s. III:10 because bedridden (tetraplegic and anarthric) at 72 and survived until 78 years. Lower limbs show marked hyperreflexia in most individuals with occasional involvement of the upper limbs. 
+Patients display a spastic gait and have frequent falls. Babinski sign is usually present of indifferent. Less overt cerebellar signs with slightly affected rapid alternating movements and finger-to-nose tests. Sensory system is intact. No hearing or visual loss. No dementia reported in the family. Nerve conduction studies normal. Electroencephalogram did not show any epileptic discharges, but did show a diffuse slowing of electrical activity. Impotence, bladder incontinence, constipation or fecal incontinence, decreased sweating, and orthostatic hypotension. 
+IV:13 had severe episodic temperature dysregulation leading to drops in temperature to as low as 32 degC. Average age of death: 62 years. 
+Brain MRI of IV:4 is representative of those seen in other family members – fluid-attenuated inversion recovery images show severe and confluent abnormalities of the white matter, even more pronounced in the posterior areas, and no significant cortical atrophy or ventriculomegaly. Spinal cord has consistently shown severe atrophy throughout. 
+Bladder/bowel disturbances, lower limb weakness, orthostatic hypotension, impotence, decreased sweating, temperature dysregulation, ataxia, MRI showing leukodystrophy, lower limb hyperreflexia with occasional upper limb involvement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedigree II - Patient 2: Sex: Male; + family history; 55 yo age of onset, 57 age at examination; + autonomic disturbance, + pyramidal signs, + ataxia; Cognitive impairment +MoCA 21 
+Pedigree II - Patient 3: Sex: Male; + family history; 52 yo age of onset; + autonomic disturbance; + pyramidal signs; + ataxia; Cognitive impairment +MMSE15 </t>
   </si>
 </sst>
 </file>
@@ -752,7 +758,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -768,6 +774,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1110,7 +1119,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B3" s="2">
         <v>5</v>
@@ -1128,12 +1137,12 @@
         <v>16</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B4" s="2">
         <v>5</v>
@@ -1151,12 +1160,12 @@
         <v>16</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B5" s="2">
         <v>5</v>
@@ -1174,12 +1183,12 @@
         <v>16</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B6" s="2">
         <v>5</v>
@@ -1197,12 +1206,12 @@
         <v>16</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B7" s="2">
         <v>5</v>
@@ -1217,15 +1226,15 @@
         <v>169456</v>
       </c>
       <c r="F7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>36</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B8" s="2">
         <v>5</v>
@@ -1240,15 +1249,15 @@
         <v>340785</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B9" s="2">
         <v>5</v>
@@ -1266,12 +1275,12 @@
         <v>16</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B10" s="2">
         <v>5</v>
@@ -1289,12 +1298,12 @@
         <v>16</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B11" s="2">
         <v>5</v>
@@ -1312,12 +1321,12 @@
         <v>16</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B12" s="2">
         <v>5</v>
@@ -1334,7 +1343,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B13" s="2">
         <v>5</v>
@@ -1352,12 +1361,12 @@
         <v>16</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B14" s="2">
         <v>5</v>
@@ -1375,12 +1384,12 @@
         <v>16</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B15" s="2">
         <v>5</v>
@@ -1397,7 +1406,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B16" s="2">
         <v>5</v>
@@ -1415,12 +1424,12 @@
         <v>16</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B17" s="2">
         <v>5</v>
@@ -1435,15 +1444,15 @@
         <v>672515</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B18" s="2">
         <v>5</v>
@@ -1458,12 +1467,12 @@
         <v>4365976</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B19" s="2">
         <v>5</v>
@@ -1478,12 +1487,12 @@
         <v>4366000</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B20" s="2">
         <v>5</v>
@@ -1500,7 +1509,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B21" s="2">
         <v>5</v>
@@ -1517,7 +1526,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B22" s="2">
         <v>5</v>
@@ -1532,15 +1541,15 @@
         <v>608833</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B23" s="2">
         <v>5</v>
@@ -1555,15 +1564,15 @@
         <v>474998</v>
       </c>
       <c r="F23" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="G23" s="5" t="s">
         <v>100</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B24" s="2">
         <v>5</v>
@@ -1580,7 +1589,7 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B25" s="2">
         <v>5</v>
@@ -1595,15 +1604,15 @@
         <v>250000</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B26" s="2">
         <v>5</v>
@@ -1618,12 +1627,12 @@
         <v>275347</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B27" s="2">
         <v>5</v>
@@ -1641,12 +1650,12 @@
         <v>16</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B28" s="2">
         <v>5</v>
@@ -1664,12 +1673,12 @@
         <v>16</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B29" s="2">
         <v>5</v>
@@ -1687,12 +1696,12 @@
         <v>16</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B30" s="2">
         <v>5</v>
@@ -1710,12 +1719,12 @@
         <v>16</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B31" s="2">
         <v>5</v>
@@ -1733,12 +1742,12 @@
         <v>16</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B32" s="2">
         <v>5</v>
@@ -1756,12 +1765,12 @@
         <v>16</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B33" s="2">
         <v>5</v>
@@ -1779,12 +1788,12 @@
         <v>16</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B34" s="2">
         <v>5</v>
@@ -1801,7 +1810,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B35" s="2">
         <v>5</v>
@@ -1818,7 +1827,7 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B36" s="2">
         <v>5</v>
@@ -1833,12 +1842,12 @@
         <v>156734</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B37" s="2">
         <v>5</v>
@@ -1855,7 +1864,7 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B38" s="2">
         <v>5</v>
@@ -1870,12 +1879,12 @@
         <v>59651</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B39" s="2">
         <v>5</v>
@@ -1893,12 +1902,12 @@
         <v>16</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B40" s="2">
         <v>5</v>
@@ -1910,12 +1919,12 @@
         <v>126903760</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B41" s="2">
         <v>5</v>
@@ -1927,12 +1936,12 @@
         <v>126896451</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B42" s="2">
         <v>5</v>
@@ -1981,7 +1990,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>15</v>
       </c>
@@ -1991,16 +2000,16 @@
       <c r="C2" s="2">
         <v>16</v>
       </c>
-      <c r="E2" s="5" t="s">
-        <v>19</v>
+      <c r="E2" s="6" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C3" s="2">
         <v>31</v>
@@ -2009,15 +2018,15 @@
         <v>45</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C4" s="2">
         <v>3</v>
@@ -2026,197 +2035,197 @@
         <v>43</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C5" s="2">
         <v>3</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>40</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>44</v>
-      </c>
       <c r="E7" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>40</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C9" s="2">
         <v>4</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C10" s="2">
         <v>4</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>40</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>82</v>
-      </c>
       <c r="E16" s="5" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C17" s="2">
         <v>3</v>
       </c>
       <c r="D17" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="E17" s="5" t="s">
         <v>185</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C19" s="2">
         <v>5</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C21" s="2">
         <v>32</v>
@@ -2224,10 +2233,10 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C22" s="2">
         <v>1</v>
@@ -2236,37 +2245,37 @@
         <v>52</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C25" s="2">
         <v>1</v>
@@ -2275,64 +2284,64 @@
         <v>34</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="E29" s="5" t="s">
         <v>201</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C31" s="2">
         <v>12</v>
@@ -2341,69 +2350,69 @@
         <v>45</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C32" s="2">
         <v>8</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C38" s="2">
         <v>2</v>
@@ -2412,23 +2421,23 @@
         <v>58</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C40" s="2">
         <v>6</v>
@@ -2437,41 +2446,41 @@
         <v>44</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="195" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>182</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>183</v>
       </c>
       <c r="C41" s="2">
         <v>6</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="E41" s="5" t="s">
-        <v>192</v>
+        <v>189</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C42" s="2">
         <v>6</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>
@@ -2513,528 +2522,528 @@
         <v>15</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>21</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="D3" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="5" t="s">
         <v>30</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B4" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>49</v>
-      </c>
       <c r="E4" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B6" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="D6" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="D7" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="5" t="s">
         <v>58</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>54</v>
-      </c>
       <c r="D8" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C9" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="E9" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>54</v>
-      </c>
       <c r="D11" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C16" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="E16" s="5" t="s">
         <v>89</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="B17" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="C17" s="5" t="s">
+      <c r="D17" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="B19" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="C19" s="5" t="s">
+      <c r="D19" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="E19" s="5" t="s">
         <v>89</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B21" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E21" s="5" t="s">
         <v>179</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C22" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B23" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C23" s="5" t="s">
-        <v>54</v>
-      </c>
       <c r="D23" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C24" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E24" s="5" t="s">
         <v>89</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B25" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C25" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="D25" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B26" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>105</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B27" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="D27" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>127</v>
-      </c>
       <c r="E27" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C29" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="E29" s="5" t="s">
         <v>204</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B30" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C30" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C30" s="5" t="s">
-        <v>54</v>
-      </c>
       <c r="D30" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B31" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="C31" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="D31" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E31" s="5" t="s">
         <v>131</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="E31" s="5" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B32" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="C32" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="D32" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="E32" s="5" t="s">
         <v>147</v>
-      </c>
-      <c r="E32" s="5" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B35" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C35" s="5" t="s">
         <v>105</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B37" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="C37" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="D37" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B40" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="C40" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="C40" s="5" t="s">
-        <v>159</v>
-      </c>
       <c r="D40" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B41" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="C41" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="C41" s="5" t="s">
-        <v>159</v>
-      </c>
       <c r="D41" s="2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="D42" s="2" t="s">
         <v>214</v>
-      </c>
-      <c r="B42" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="C42" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>216</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
the Excel sheet was not completely up to date
updated and testing again now
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\Krizchelle\ADLD Patient Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9672A1B2-89B3-4306-8B8A-1008DA86F5EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD5A6A61-A42E-4F79-9F67-4C137756E9BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Molecular" sheetId="4" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="220">
   <si>
     <t>Item name</t>
   </si>
@@ -118,9 +118,6 @@
     <t>Sweden</t>
   </si>
   <si>
-    <t>Bladder symptoms, constipation, postural hypotention, erectile dysfunction , pyramidal signs, Ataxia, NCS: Normal, SEP:Normal: , MRI showing leukodystrophy, normal cognition</t>
-  </si>
-  <si>
     <t>10.1002/humu.22348, 10.1007/s10048-010-0269-y, PMC8133955, 10.3174/ajnr.A1354, 10.1002/ajmg.b.30342, 10.1002/ana.24452</t>
   </si>
   <si>
@@ -172,12 +169,6 @@
     <t>40.5 ± 4.9</t>
   </si>
   <si>
-    <t>Bladder symptoms, constipation, postural hypotention, dry skin, pyramidal signs, Ataxia, VEP: Normal, NCS: Normal, SEP: Pathological , MRI showing leukodystrophy, increased symptoms with infection</t>
-  </si>
-  <si>
-    <t>Bowel/bladder dysfunction, impotence, orthostatic hypotention, decreased sweating, pyramidal signs, ataxia, MRI showing leukodystrophy, spastic paralysis, posterior column dysfunction, Babinski signs</t>
-  </si>
-  <si>
     <t>10.1002/humu.22348, 10.1007/s10048-010-0269-y, PMC8133955, 10.3174/ajnr.A1354, 10.1002/ana.24452</t>
   </si>
   <si>
@@ -259,12 +250,6 @@
     <t>Microhomology of "GG"</t>
   </si>
   <si>
-    <t>Bladder symptoms, constipation, erectile dysfunction, pyramidal signs, Ataxia, MMT: 23, distal sensory loss clinically, NCS: Normal, MRI showing leukodystrophy, postural tremor, perkinsonism, Levodopa responsive</t>
-  </si>
-  <si>
-    <t>Bladder symptoms, postural hypotension, heat intolerance, fecal incontinnence, pyramidal signs, ataxia, MMT: 24, 26, NCS: Normal, MRI showing leukodystrophy</t>
-  </si>
-  <si>
     <t>ADLD_dup_11</t>
   </si>
   <si>
@@ -595,33 +580,21 @@
     <t>34, 33, 37, 32</t>
   </si>
   <si>
-    <t>Late urinary urgency, dysarthria, speech apraxia and dysphafia, MRI showing leukodystrophy, asymmetrical spastic weakness of upper and lower extremities, decreased dexterity upper limb spasticity, dyspnea likely from neuromuscular weakness, neurological defects reported to be worsened by environmental heat, Additional details from three patients also listed out in Master Excel but too lengthy in the current organization of the website to paste here</t>
-  </si>
-  <si>
     <t>Canada; Northern European</t>
   </si>
   <si>
     <t>Urinary urgency and incontinence, ataxia, MRI showing leukodystrophy, slowly progressive spasticity of lower, Sex: Male, Age at symptom onset: 52, Ethnicity: Northern European, Affect: Chronic anxiety, Oral motor control and atriculation: Speech was normal, Eye and extraocular movement examination: Fine end-point nystagmus on lateral gaze, interrupted saccades, in vertical and horizontal planes, Motor examination: Tremor of lower extremities, spasticity, and cerebellar deficits, DTRs/plantar responses: Spastic in all limbs with lower limb clonus; positive Hoffman response, Sensory examination: Normal, Autonomic nervous system: late urinary urgency adn incontinence, EMG/NCV: Normal, Family history and inheritance patterns: Positive/autosomal dominant, Comorbidities: Hypertension, GERD, and degenerative joint diseaselimbs, fine motor difficulty, fine end point nystagmus on left and right lateral gaze, leg cramps, snout reflex</t>
   </si>
   <si>
-    <t>Early orthostatix intolerance, urinary urgency, ataxia, soft "breathy" and halting voice and dysphagia, MRI showing leukodystrophy, hand tremor, voice difficulties, neurological deficits worsened with respiratory infection, Affect: Normal, Oral motor control and atriculation: Soft "breathy" and halting voice and dysphagia, Eye and extraocular movement examination: normal, Motor examination: Head and hand tremor (asymmetrical), incoordination and spastic and ataxic gait, and weakness of lower extremeties, DTRs/plantar responses: Brisk with clonus/extensor, Sensory examination: Normal, Autonomic nervous system: Early orthostatic intolerance and urinary urgency, EMG/NCV: NA, Family history and inheritance patterns: Negative, Comorbidities: Migraines, gout, and dyslipidemia</t>
-  </si>
-  <si>
     <t>55, 52, 50</t>
   </si>
   <si>
-    <t>Negative family history, + autonomic disturbance, + pyramidal signs, + Ataxia, Cognitive impairment +MMSE23, MRI findings with MCP lesion</t>
-  </si>
-  <si>
     <t>Pedigree I - Patient I</t>
   </si>
   <si>
     <t>Pedigree II - Patient 2, Pedigree II - Patient 3, Pedigree III - Patient 4</t>
   </si>
   <si>
-    <t>Symptoms listed in Master excel from the different individuals while we finalize formating of the database</t>
-  </si>
-  <si>
     <t>F2-1, F2-2, F2-3</t>
   </si>
   <si>
@@ -643,9 +616,6 @@
     <t>48, 50, 48, 42</t>
   </si>
   <si>
-    <t>Urinary urgency, ejaculatory failure, orthostatic intolerance, selective noradreneric failure, isolated cardiovascular sympathetic impairment, pyramidal signs, ataxia, MRI showing leukodystrophy, many additional information for the IV family that is too lengthy for the current version of the website</t>
-  </si>
-  <si>
     <t>Giorgio 2013, Guaraldi 2011, Terlizzi et al. 2016</t>
   </si>
   <si>
@@ -662,9 +632,6 @@
   </si>
   <si>
     <t>China</t>
-  </si>
-  <si>
-    <t>Dificulty using her hands with involuntary movement, gait imbalance, urinary incontinence, constipation, speech slowly and mild inarticulate speech, neurological - postural tremor of all extremities, increasing frequency and intensity of involuntary movement when keeping arms flat or when in a standing posture, slightly increased muscle tone adn mild spasticity in the lower limbs, MMSE normal, MRI showed diffuse and symmetrical T2-hyperintense lesions in WM with less affected perventricular rims, mild withering of the cerebellum, brain stem, cerebrum, and difuse spinal cord atrophy family history - father and elder sister had similar gait impairment at least 10 years before heath and brother had several years' history of autonomic symptoms and gait disturbance and nephew has diffiulty walking</t>
   </si>
   <si>
     <t>Predicted junction</t>
@@ -695,6 +662,48 @@
   <si>
     <t xml:space="preserve">Pedigree II - Patient 2: Sex: Male; + family history; 55 yo age of onset, 57 age at examination; + autonomic disturbance, + pyramidal signs, + ataxia; Cognitive impairment +MoCA 21 
 Pedigree II - Patient 3: Sex: Male; + family history; 52 yo age of onset; + autonomic disturbance; + pyramidal signs; + ataxia; Cognitive impairment +MMSE15 </t>
+  </si>
+  <si>
+    <t>Sex: Male; Onset: 45 year; Autonomic symptoms: Bladder symptoms, constipation, postural hypotension, erectile dysfunction; Pyramidal signs: +; Ataxia: +; Cognition: Normal; Neurophysiological studies: NCS: normal, SEP: normal; MRI showing leukodystrophy: +; Includes 31 affected family members; Bladder symptoms, constipation, postural hypotention, erectile dysfunction , pyramidal signs, Ataxia, NCS: Normal, SEP:Normal: , MRI showing leukodystrophy, normal cognition</t>
+  </si>
+  <si>
+    <t>Sex: Male; Onset: 43 year; Autonomic symptoms: Bladder symptoms, constipation, postural hypotension, dry skin; Pyramidal signs: +; Ataxia: +; Cognition: Normal; Neurophysiological studies: VEP: normal, NCS: normal; SEP: pathological; MRI showing leukodystrophy: +; Other symptoms/signs: Increased symptoms with infection; Includes 3 affected family members // Bladder symptoms, constipation, postural hypotention, dry skin, pyramidal signs, Ataxia, VEP: Normal, NCS: Normal, SEP: Pathological , MRI showing leukodystrophy, increased symptoms with infection</t>
+  </si>
+  <si>
+    <t>20 individuals in this family were misdiagnosed as having chronic progressive MS.  \Early autonomic dysfunction. CT/MRI scans illustrate a widespread symmetrical demyelination of the white matter, normal immunoglobulin levels in cerebrospinal fluid, no pathological indication of brain inflammation has been found. Five generations of the ADLD pedigree involved. Disease onset mean age: 40.5 +- 4.9 years, n = 16. The earliest symptoms usually involve abnormalities of the autonomic nervous system, such as bowel/bladder dysfunction, impotence, orthostatic hypotension and decreased sweating. These symptoms precede others by several years and are followed by loss of fine motor skills. Nerve conduction velocities performed on three affected individuals were normal. Spastic paralysis and posterior column dysfunction occur in 88% of these patients, and 81% exhibit Babinski signs. Exhibit cerebellar signs. For instance, nystagmus is present in 69% of the individuals, and all patients experience ataxia. // Bowel/bladder dysfunction, impotence, orthostatic hypotention, decreased sweating, pyramidal signs, ataxia, MRI showing leukodystrophy, spastic paralysis, posterior column dysfunction, Babinski signs | Ireland: 47-year-old man with 6-year history of autonomic dysfunction; Progressive fatigue, gait ataxia, falls, dysarthria, urinary frequency, and urinary urgency; Examination showed gait ataxia and bilateral past-pointing; Neurological signs progressed over time; MRI demonstrated widespread diffuse white-matter disease with interval radiologic progression on repeat imaging; Slowly progressive multisystem neurological dysfunction consistent with ADLD caused by LMNB1 duplication; First genetically confirmed Irish case reported. | 1/58/F: Constipation for many years before neurologic symptoms. Fine motor difficulty starting in her 40s. Progressive gait difficulty, hand numbness, urinary frequency, and incontinence. Ataxia, spastic paraparesis, dysarthria, dysmetria, head titubation, hyperreflexia, sensory loss, orthostatic hypotension, confusion, lethargy, and mild dementia. Eventually wheelchair-bound and bedridden. CT/MRI showed severe diffuse symmetric white-matter disease, greatest in frontoparietal regions, with cerebellar involvement and ventricular enlargement. | 2/50/F: 15-year progressive neurologic illness. Ataxia, weakness, sensory symptoms, urinary dysfunction, constipation, decreased sweating, orthostatic light-headedness, visual complaints, and hearing impairment. MRI showed severe diffuse cerebral white-matter abnormalities with ventricular enlargement. CT showed diffuse frontoparietal white-matter lucencies. | 3/60/F: 7-year history of progressive ataxia and weakness. Urinary dysfunction, constipation, decreased sweating, visual complaints, and hearing impairment. MRI showed moderate diffuse cerebral white-matter disease with mild ventricular enlargement. CT showed mild frontoparietal-predominant white-matter changes. | 4/53/M: 20-year progressive illness. Ataxia, weakness, sensory symptoms, urinary dysfunction, constipation, decreased sweating, orthostatic symptoms, hearing impairment, and impotence. MRI showed moderate cerebral white-matter abnormalities with cerebellar and brainstem involvement. CT showed mild frontoparietal white-matter disease. | 5/56/M: 18-year progressive illness. Ataxia, weakness, sensory symptoms, urinary dysfunction, constipation, decreased sweating, orthostatic symptoms, visual complaints, and impotence. MRI showed severe diffuse cerebral white-matter abnormalities with cerebellar involvement and ventricular enlargement. CT showed diffuse centrum semiovale white-matter lucencies.</t>
+  </si>
+  <si>
+    <t>Bladder symptoms, constipation, erectile dysfunction, pyramidal signs, Ataxia, MMT: 23, distal sensory loss clinically, NCS: Normal, MRI showing leukodystrophy, postural tremor, perkinsonism, Levodopa responsive // Patient 1: Sex: M; Onset: 54 year; Autonomic symptoms: Bladder symptoms, constipation, erectile dysfunction; Pyramidal signs: +, Ataxia: +; Cognition: Normal; Neurophysiological studies: Distal sensory loss clinically; MRI showing leukodystrophy: +; Other symptoms/signs: Postural tremor; 4 patients were affected in the IL family over three generations. Patients in the family had an onset in their 6th decade with autonomic symptoms, pyramidal signs, and had brain MRI signs characteristic of ADLD. Patient 2: Sex: M; Onset: 50 year; Autonomic symptoms: Bladder symptoms, constipation, erectile dusfunction; Pyramidal signs: +; Ataxia: +; Cognition: MMT: 23; Neurophysiological studies: NCS: normal; MRI showing leukodystrophy: +; Other symptoms/signs: Parkinsonism, levodopa responsive, no tremor; 4 patients were affected in the IL family over three generations. Patients in the family had an onset in their 6th decade with autonomic symptoms, pyramidal signs, and had brain MRI signs characteristic of ADLD.</t>
+  </si>
+  <si>
+    <t>Bladder symptoms, postural hypotension, heat intolerance, fecal incontinnence, pyramidal signs, ataxia, MMT: 24, 26, NCS: Normal, MRI showing leukodystrophy // Sex: Female; Onset: 53 year; Autonomic symptoms: Bladder symptoms, postural hypotension, heat intolerance; Pyramidal signs: +; Ataxia: +; Cognition: MMT: 24; Neurophysiological studies: NCS: normal; MRI showing leukodystrophy: +; 4 patients were affected in the DE family over two generations. Patients in the family had an onset in their 6th decade with autonomic symptoms, pyramidal signs, and had brain MRI signs characteristic of ADLD. | Patient 2: Sex: Female; Onset: 58 year; Autonomic symptoms: Bladder symptoms, fecal incontinence; Pyramidal signs: +; Ataxia: unknown; Cognition: MMT: 26; Neurophysiological studies: NCS: normal; MRI showing leukodystrophy: +; 4 patients were affected in the DE family over two generations. Patients in the family had an onset in their 6th decade with autonomic symptoms, pyramidal signs, and had brain MRI signs characteristic of ADLD.</t>
+  </si>
+  <si>
+    <t>F2-1: Sex: Male; Negative family history suggestive of LD; Comorbidities: osteoarthritis; No dysautonomic symptoms; No documented orthostatic hypotension; Neurological examination showed difficulty walking attributed to osteoarthritis; No neurodegeneration suggestive of LD; No MRI evidence of LD; Father of F2-2, grandfather of F2-3. | F2-2: Sex: Female; Negative family history suggestive of LD; Comorbidities: depression, anxiety; Presence of dysautonomic symptoms; No documented orthostatic hypotension; Neurological examination showed nystagmus, hyperreflexia and spasticity; No neurodegeneration suggestive of LD; No MRI evidence of LD; Daugther of F2-1, mother of F2-3 | F2-3: Sex: Female; Negative family history suggestive of LD; Comorbidities: speech delay, learning difficulties, behavioral difficulties; Dysautonomic symptoms present; No documented orthostatic hypotension; Neurological examination showed lower limbs hyperreflexia with left plantar unresponsiveness; No neurodegeneration suggestive of LD; No MRI evidence of LD; Daughter of F2-2, granddaughter of F2-1</t>
+  </si>
+  <si>
+    <t>Late urinary urgency, dysarthria, speech apraxia and dysphafia, MRI showing leukodystrophy, asymmetrical spastic weakness of upper and lower extremities, decreased dexterity upper limb spasticity, dyspnea likely from neuromuscular weakness, neurological defects reported to be worsened by environmental heat. | DEL3-1: Sex: Female; Age at symptom onset: 37; Ethnicity: Northern European/Native American; Affect: Depressed mood; Oral motor control and atriculation: Muffled voice, unilateral facial weakness, and drooling; Eye and extraocular movement examination: Normal dilated examination, Saccadic intrusion; Motor examination: Asymmetrical spastic weakness of upper and lower extremities; DTRs/plantar responses: Lower extremity clonus/extensor; Sensory examination: Normal; Autonomic nervous system: Normal by history and laboratory testing; EMG/NCV: Normal; Family history and inheritance patterns: Positive/autosomal dominant; Comorbidities: Neurologic deficity reported to be worsened by environmental heat | DEL3-2: Sex: Female; Age at symptom onset: 34; Ethnicity: Northern European/Native American; Affect: Normal; Oral motor control and atriculation: Speech apraxia and dysphagia; Eye and extraocular movement examination: Optic disk pallor, limited up-gaze and sacadic intrusion; Motor examination: Asymmetrical (left &gt; right) spastic weakness of upper and lower extremities; DTRs/plantar responses: Brisk; Sensory examination: Normal; Autonomic nervous system: Normal by history; EMG/NCV: L peroneal entrapment neuropathy; Family history and inhertance patterns: Positive/autosomal dominant; Comorbidities: Dyspnea likely from neuromusclar weakness; L leg pain likely from peroneal neuropathy | DEL3-3: Sex: Male; Age at symptom onset: 32; Ethnicity: Northern European/Native American; Affect: Pseudobulbar affect; Oral motor control and atriculation: Dysarthria; Eye and extraocular movement examination: Normal; Motor examination: Decreased dexterity upper limb spasticity and asymmetrical weakness of upper and lower limbs (right &gt; left); DTRs/plantar responses: Brisk/extensor; Sensory examination: Normal; Autonomic nervous system: Late urinary urgency; EMG/NCV: NA; Family history and inheritance patterns: Positive/autosomal dominant; Comorbidities: Neurological deficits resported to be worsened by environmental heat</t>
+  </si>
+  <si>
+    <t>F1-1: Sex: Male; Negative family history suggestive of LD; Comorbidities: gout, diabetes, Parkinson, axonal sensorimotor polyneuropathy; Dysautonomic symptoms present; Orthostatic hypotension present; Neurological examination consistent with Parkinson and polyneuropathy; No neurodegeneration suggestive of LD; No MRI evidence of LD; Sibling of F1-2, father of F1-3, grandfather of F1-5 | F1-2: Sex: Male; Negative family history suggestive of LD; Comorbidities: hypothyroidism, sensorineural hearing loss, Meniere, posterior vitreous detachment, hypertension, essential tremor, mild cognitive impairment, irritable bowel syndrome; Negative for dysautonomic symptoms; No documented orthostatic hypotension; Neurological examination showed slightly unsteady gait and the inability to perform the tandem gait; No neurodegeneration suggestive of LD; No MRI evidence of LD; Sibling to F1-1, father of F1-4 | F1-3: Sex: Female; Negative for family history suggestive of LD; Comorbidities: asthma, irritable bowel syndrome, migraines, goiter, erythema nodosum, chronic pain, carpal tunnel syndrome; Dysautonomic symptoms present; No documented orthostatic hypotension; Neurological examination showed slightly slow tongue movements, mild weakness in shoulder abduction, slightly slow fine finger movements and an absent right ankle jerk; No neurodegeneration suggestive of LD; No MRI evidence of LD; Daughter of F1-1, Mother of F1-5 | F1-4: Sex: Male; Negative family history suggestive of LD; Comorbidities: hypothyroidism, depression, back pain; Dysautonomic symptoms present; No documented orthostatic hypotension; Neurological examination showed brisk reflexes, 3-5 beats of clonus, down going plantar, decreased sensation on the left L5-S1 distribution, slow and hesitant gait; No neurodegeneration suggestive of LD; No MRI evidence of LD; Son of F1-2 | F1-5: Sex: Male; Negative family history suggestive of LD; Comorbidities: failure to thrive, microcephaly, global developmental delay, autistic spectrum disorder, learning difficulties, mild dysmorphic facial features; No dysautonomic symptoms; No documented orthostatic hypotension; Neurological examination normal; No neurodegeneration suggestive of LD; No MRI evidence of LD; Son of F1-3, grandson of F1-1</t>
+  </si>
+  <si>
+    <t>Sex: Male; Positive family history suggestive of LD (mother and maternal grandmother with neurological regression around 30 years and death a few years later); Comorbidities: neurological sequelae from MVA at age 31; Dysautonomic symptoms present; Documented orthostatic hypotension present; Neurological examination showed spastic gait, dysdiadokokinesia on the left side, brisk deep tendon reflexes, clonus, Babinski, dysautonomia at age 33; Neurodegeneration suggestive of LD present: bed ridden, no sphincter control, gastronomy at age 39; Presence of MRI evidence of LD</t>
+  </si>
+  <si>
+    <t>F3-1: Sex: Female; Negative family history suggestive of LD; No comorbidities; No dysautonomic symptoms; No documented orthostatic hypotension; Neurological examination unremarkable; No neurodegeneration suggestive of LD; No MRI evidence of LD; Mother of F3-2 | F3-2: Sex: Female; Negative family history suggestive of LD; Comorbidities: chronic dysuria and UTIs, refractory depression, hypothyroidism, hyperlipidemia, panhypopituitarism, vitamin B12 deficiency, ankylosing spondylitis, fibromyalgia; Dysautonomic symptoms present; Documented orthostatic hypotension present; Neurological examination showed gait disturbance; Mild hyperreflexia; No neurodegeneration suggestive of LD; No MRI evidence of LD; Daughter of F3-1</t>
+  </si>
+  <si>
+    <t>DEL1-1: Sex: Male; Age at symptom onset: 34; Ethnicity: East Asian; Affect: Normal; Oral motor control and atriculation: Soft "breathy" and halting voice and dysphagia; Eye and extraocular movement examination: normal; Motor examination: Head and hand tremor (asymmetrical), incoordination and spastic and ataxic gait, and weakness of lower extremeties; DTRs/plantar responses: Brisk with clonus/extensor; Sensory examination: Normal; Autonomic nervous system: Early orthostatic intolerance and urinary urgency; EMG/NCV: NA; Family history and inheritance patterns: Negative; Comorbidities: Migraines, gout, and dyslipidemia | Pedigree IV-Patient 5: Sex: Female; Postive family history; 43 yo age of onset; Negative autonomic disturbance; Postive for pyramidal signs; Positive for ataxia; Cognitive impairment +MMSE 9 | Pedigree IV-Patient 6: Sex: Male; Positive family history; 34 yo age of onset; Negative autonomic disturbance; Postive for pyramidal signs; Positive for ataxia; Cognitive impairment +MoCA 10</t>
+  </si>
+  <si>
+    <t>Urinary urgency, ejaculatory failure, orthostatic intolerance, selective noradreneric failure, isolated cardiovascular sympathetic impairment, pyramidal signs, ataxia, MRI showing leukodystrophy | Cardiovascular reflexes and pharmacological assessment indicated a selective sympathetic failure, sparing cardiovagal function. Microneurography revealed absent sympathetic activity. The evaluation of autonomic innervation of skin annexes showed severely depleted and morphologically abnormal noradrenergic dopamine-β-hydroxylase (DβH) immunoreactive fibres with preserved cholinergic vasoactive intestinal polypeptide (VIP) immunoreactive fibres. | IV11: Sex: Female; Sibling to IV11 and IV12; Age of onset 50; Clinical signs at first evaluation at age 53 - autonomic symptoms: bowel/bladder dysfunction, OH, cerebellar signs: ataxia; pyramidal signs: brisk tendon reflexes; psuedobulbar signs absent; detailed clinical progression listed in paper | IV10: Sex: Male; Sibling to IV10 and IV12; Age of onset 48; clinical signs at first evaluation at age 50 - autonomic symptoms: bowel/bladder dysfunction, impotence, OH; cerebellar signs: nystagmus, dysmetria, ataxia; pyramidal signs: brisk tendon reflexes, pseudobulbar signs absent; detailed clinical progression listed in paper | IV12: Sex: Male; Sibling to IV10 and IV11; age at onset: 42; clinical signs at first evaluation at 44 years old - autonomic symptoms: bladder dysfunction, impotence, OH; cerebellar signs: action tremor, ataxia; pyramidal signs: brisk tendon reflexes, pseudobulbar signs absent; detailed clinical progression listed in paper</t>
+  </si>
+  <si>
+    <t>Proband II-4: Sex: Female; Difficulty using her hands with involuntary movement, gait imbalance, urinary incontinence, constipation, speech slowly and mild inarticulate speech; Neurological - postural tremor of all extremities, increasing frequency and intensity of involuntary movement when keeping arms flat or when in a standing posture, slightly increased muscle tone and mild spasticity in the lower limbs, MMSE normal, MRI showed diffuse and symmetrical T2-hyperintense lesions in WM with less affected perventricular rims, mild withering of the cerebellum, brain stem, cerebrum, and difuse spinal cord atrophy; Family history - father and elder sister had similar gait impairment at least 10 years before heath and brother had several years' history of autonomic symptoms and gait disturbance and nephew has diffiulty walking</t>
+  </si>
+  <si>
+    <t>Pedigree I - Patient 1: Sex: Female; Negative family history; 44 yo age of onset; + autonomic disturbance; + pyramidal signs; + Ataxia; Cognitive impairment +MMSE23; MRI findings with MCP lesion</t>
   </si>
 </sst>
 </file>
@@ -1142,7 +1151,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B4" s="2">
         <v>5</v>
@@ -1160,12 +1169,12 @@
         <v>16</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" s="2">
         <v>5</v>
@@ -1183,12 +1192,12 @@
         <v>16</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B6" s="2">
         <v>5</v>
@@ -1206,12 +1215,12 @@
         <v>16</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B7" s="2">
         <v>5</v>
@@ -1226,15 +1235,15 @@
         <v>169456</v>
       </c>
       <c r="F7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>35</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B8" s="2">
         <v>5</v>
@@ -1249,15 +1258,15 @@
         <v>340785</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B9" s="2">
         <v>5</v>
@@ -1275,12 +1284,12 @@
         <v>16</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B10" s="2">
         <v>5</v>
@@ -1298,12 +1307,12 @@
         <v>16</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B11" s="2">
         <v>5</v>
@@ -1321,12 +1330,12 @@
         <v>16</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="B12" s="2">
         <v>5</v>
@@ -1343,7 +1352,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B13" s="2">
         <v>5</v>
@@ -1361,12 +1370,12 @@
         <v>16</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B14" s="2">
         <v>5</v>
@@ -1384,12 +1393,12 @@
         <v>16</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B15" s="2">
         <v>5</v>
@@ -1406,7 +1415,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="B16" s="2">
         <v>5</v>
@@ -1424,12 +1433,12 @@
         <v>16</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B17" s="2">
         <v>5</v>
@@ -1444,15 +1453,15 @@
         <v>672515</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B18" s="2">
         <v>5</v>
@@ -1467,12 +1476,12 @@
         <v>4365976</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="B19" s="2">
         <v>5</v>
@@ -1487,12 +1496,12 @@
         <v>4366000</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B20" s="2">
         <v>5</v>
@@ -1509,7 +1518,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B21" s="2">
         <v>5</v>
@@ -1526,7 +1535,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B22" s="2">
         <v>5</v>
@@ -1541,15 +1550,15 @@
         <v>608833</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B23" s="2">
         <v>5</v>
@@ -1564,15 +1573,15 @@
         <v>474998</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B24" s="2">
         <v>5</v>
@@ -1589,7 +1598,7 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B25" s="2">
         <v>5</v>
@@ -1604,15 +1613,15 @@
         <v>250000</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B26" s="2">
         <v>5</v>
@@ -1627,12 +1636,12 @@
         <v>275347</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B27" s="2">
         <v>5</v>
@@ -1650,12 +1659,12 @@
         <v>16</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B28" s="2">
         <v>5</v>
@@ -1673,12 +1682,12 @@
         <v>16</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B29" s="2">
         <v>5</v>
@@ -1696,12 +1705,12 @@
         <v>16</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B30" s="2">
         <v>5</v>
@@ -1719,12 +1728,12 @@
         <v>16</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B31" s="2">
         <v>5</v>
@@ -1742,12 +1751,12 @@
         <v>16</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B32" s="2">
         <v>5</v>
@@ -1765,12 +1774,12 @@
         <v>16</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="B33" s="2">
         <v>5</v>
@@ -1788,12 +1797,12 @@
         <v>16</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B34" s="2">
         <v>5</v>
@@ -1810,7 +1819,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="B35" s="2">
         <v>5</v>
@@ -1827,7 +1836,7 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="B36" s="2">
         <v>5</v>
@@ -1842,12 +1851,12 @@
         <v>156734</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B37" s="2">
         <v>5</v>
@@ -1864,7 +1873,7 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="B38" s="2">
         <v>5</v>
@@ -1879,12 +1888,12 @@
         <v>59651</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="B39" s="2">
         <v>5</v>
@@ -1902,12 +1911,12 @@
         <v>16</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="B40" s="2">
         <v>5</v>
@@ -1919,12 +1928,12 @@
         <v>126903760</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B41" s="2">
         <v>5</v>
@@ -1936,12 +1945,12 @@
         <v>126896451</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="B42" s="2">
         <v>5</v>
@@ -2001,7 +2010,7 @@
         <v>16</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>215</v>
+        <v>204</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -2018,12 +2027,12 @@
         <v>45</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>26</v>
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>25</v>
@@ -2035,197 +2044,197 @@
         <v>43</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>44</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C5" s="2">
         <v>3</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>43</v>
-      </c>
       <c r="E7" s="5" t="s">
-        <v>45</v>
+        <v>208</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>63</v>
       </c>
       <c r="C9" s="2">
         <v>4</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>73</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C10" s="2">
         <v>4</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>74</v>
+        <v>210</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>193</v>
+        <v>211</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C17" s="2">
         <v>3</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>185</v>
+        <v>212</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C19" s="2">
         <v>5</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>193</v>
+        <v>213</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="C21" s="2">
         <v>32</v>
@@ -2233,10 +2242,10 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="C22" s="2">
         <v>1</v>
@@ -2245,37 +2254,37 @@
         <v>52</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>40</v>
+        <v>214</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>193</v>
+        <v>215</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="C25" s="2">
         <v>1</v>
@@ -2284,64 +2293,64 @@
         <v>34</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>188</v>
+        <v>216</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C31" s="2">
         <v>12</v>
@@ -2350,69 +2359,69 @@
         <v>45</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C32" s="2">
         <v>8</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="C38" s="2">
         <v>2</v>
@@ -2421,23 +2430,23 @@
         <v>58</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="C40" s="2">
         <v>6</v>
@@ -2446,41 +2455,41 @@
         <v>44</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>190</v>
+        <v>219</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="195" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="C41" s="2">
         <v>6</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>216</v>
+        <v>205</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="C42" s="2">
         <v>6</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -2539,511 +2548,511 @@
         <v>23</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="D3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>55</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>19</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>19</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>214</v>
+        <v>203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Uploaded updated Excel and bb file
Excel file: updated names from "LN_dup_#" to "NonADLD_dup_#". Added new tab of "Evidence Summary". bb file - updated LN_dup names.
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\Krizchelle\ADLD Patient Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C16B7447-1DC4-4810-A71F-79D9D70DB06A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C72D020-47C9-4E62-9997-0FF7B23BA7BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Molecular" sheetId="4" r:id="rId1"/>
-    <sheet name="Clinical" sheetId="1" r:id="rId2"/>
-    <sheet name="Publication" sheetId="5" r:id="rId3"/>
+    <sheet name="Evidence" sheetId="6" r:id="rId2"/>
+    <sheet name="Clinical" sheetId="1" r:id="rId3"/>
+    <sheet name="Publication" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="225">
   <si>
     <t>Item name</t>
   </si>
@@ -100,9 +101,6 @@
     <t>10.1002/humu.22348, 10.1007/s10048-010-0269-y</t>
   </si>
   <si>
-    <t>Giorgio 2013, Meijer 2001</t>
-  </si>
-  <si>
     <t>10.1001/archneur.65.11.1496</t>
   </si>
   <si>
@@ -265,9 +263,6 @@
     <t>ADLD_dup_14</t>
   </si>
   <si>
-    <t>LN_dup_1</t>
-  </si>
-  <si>
     <t>Portugal</t>
   </si>
   <si>
@@ -283,12 +278,6 @@
     <t>10.1212/NXG.0000000000000305</t>
   </si>
   <si>
-    <t>LN_dup_2</t>
-  </si>
-  <si>
-    <t>LN_dup_3</t>
-  </si>
-  <si>
     <t>Nmezi et al. 2025</t>
   </si>
   <si>
@@ -298,9 +287,6 @@
     <t>Britain, England</t>
   </si>
   <si>
-    <t>LN_dup_4</t>
-  </si>
-  <si>
     <t>ADLD_del_2</t>
   </si>
   <si>
@@ -334,9 +320,6 @@
     <t>BR1</t>
   </si>
   <si>
-    <t>LN_dup_5</t>
-  </si>
-  <si>
     <t>10.1212/NXG.0000000000200261</t>
   </si>
   <si>
@@ -358,9 +341,6 @@
     <t>ADLD_del_4</t>
   </si>
   <si>
-    <t>LN_dup_6</t>
-  </si>
-  <si>
     <t>Microhomology of "GC"</t>
   </si>
   <si>
@@ -695,6 +675,45 @@
   </si>
   <si>
     <t xml:space="preserve">[PEDIGREE II - PATIENT 2] Sex: Male; + family history; 55 yo age of onset, 57 age at examination; + autonomic disturbance, + pyramidal signs, + ataxia; Cognitive impairment +MoCA 21. ... [PEDIGREE II - PATIENT 3] Sex: Male; + family history; 52 yo age of onset; + autonomic disturbance; + pyramidal signs; + ataxia; Cognitive impairment +MMSE15 </t>
+  </si>
+  <si>
+    <t>Giorgio 2013, Schuster 2011, Meijer 2008</t>
+  </si>
+  <si>
+    <t>10.1002/humu.22348, 10.1007/s10048-010-0269-y, 10.1001/archneur.65.11.1496</t>
+  </si>
+  <si>
+    <t>NonADLD_dup_1</t>
+  </si>
+  <si>
+    <t>NonADLD_dup_2</t>
+  </si>
+  <si>
+    <t>NonADLD_dup_3</t>
+  </si>
+  <si>
+    <t>NonADLD_dup_4</t>
+  </si>
+  <si>
+    <t>NonADLD_dup_5</t>
+  </si>
+  <si>
+    <t>NonADLD_dup_6</t>
+  </si>
+  <si>
+    <t>Publications</t>
+  </si>
+  <si>
+    <t>Literature case labels</t>
+  </si>
+  <si>
+    <t>Multigenerational families</t>
+  </si>
+  <si>
+    <t>Estimated unique affected individuals</t>
+  </si>
+  <si>
+    <t>Deduplication status</t>
   </si>
 </sst>
 </file>
@@ -1062,7 +1081,7 @@
   <dimension ref="A1:G42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.5703125" style="2" customWidth="1"/>
     <col min="2" max="2" width="6.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.5703125" style="2" bestFit="1" customWidth="1"/>
@@ -1119,7 +1138,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B3" s="2">
         <v>5</v>
@@ -1137,12 +1156,12 @@
         <v>16</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B4" s="2">
         <v>5</v>
@@ -1160,12 +1179,12 @@
         <v>16</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B5" s="2">
         <v>5</v>
@@ -1183,12 +1202,12 @@
         <v>16</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B6" s="2">
         <v>5</v>
@@ -1206,12 +1225,12 @@
         <v>16</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B7" s="2">
         <v>5</v>
@@ -1226,15 +1245,15 @@
         <v>169456</v>
       </c>
       <c r="F7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>34</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B8" s="2">
         <v>5</v>
@@ -1249,15 +1268,15 @@
         <v>340785</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B9" s="2">
         <v>5</v>
@@ -1275,12 +1294,12 @@
         <v>16</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B10" s="2">
         <v>5</v>
@@ -1298,12 +1317,12 @@
         <v>16</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B11" s="2">
         <v>5</v>
@@ -1321,12 +1340,12 @@
         <v>16</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B12" s="2">
         <v>5</v>
@@ -1343,7 +1362,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B13" s="2">
         <v>5</v>
@@ -1361,12 +1380,12 @@
         <v>16</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B14" s="2">
         <v>5</v>
@@ -1384,12 +1403,12 @@
         <v>16</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B15" s="2">
         <v>5</v>
@@ -1406,7 +1425,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>75</v>
+        <v>214</v>
       </c>
       <c r="B16" s="2">
         <v>5</v>
@@ -1424,12 +1443,12 @@
         <v>16</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B17" s="2">
         <v>5</v>
@@ -1444,15 +1463,15 @@
         <v>672515</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>81</v>
+        <v>215</v>
       </c>
       <c r="B18" s="2">
         <v>5</v>
@@ -1467,12 +1486,12 @@
         <v>4365976</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>82</v>
+        <v>216</v>
       </c>
       <c r="B19" s="2">
         <v>5</v>
@@ -1487,12 +1506,12 @@
         <v>4366000</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>86</v>
+        <v>217</v>
       </c>
       <c r="B20" s="2">
         <v>5</v>
@@ -1509,7 +1528,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="B21" s="2">
         <v>5</v>
@@ -1526,7 +1545,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B22" s="2">
         <v>5</v>
@@ -1541,15 +1560,15 @@
         <v>608833</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B23" s="2">
         <v>5</v>
@@ -1564,15 +1583,15 @@
         <v>474998</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>98</v>
+        <v>218</v>
       </c>
       <c r="B24" s="2">
         <v>5</v>
@@ -1589,7 +1608,7 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="B25" s="2">
         <v>5</v>
@@ -1604,15 +1623,15 @@
         <v>250000</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>106</v>
+        <v>219</v>
       </c>
       <c r="B26" s="2">
         <v>5</v>
@@ -1627,12 +1646,12 @@
         <v>275347</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="B27" s="2">
         <v>5</v>
@@ -1650,12 +1669,12 @@
         <v>16</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="B28" s="2">
         <v>5</v>
@@ -1673,12 +1692,12 @@
         <v>16</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="B29" s="2">
         <v>5</v>
@@ -1696,12 +1715,12 @@
         <v>16</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="B30" s="2">
         <v>5</v>
@@ -1719,12 +1738,12 @@
         <v>16</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="B31" s="2">
         <v>5</v>
@@ -1742,12 +1761,12 @@
         <v>16</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="B32" s="2">
         <v>5</v>
@@ -1765,12 +1784,12 @@
         <v>16</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="B33" s="2">
         <v>5</v>
@@ -1788,12 +1807,12 @@
         <v>16</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="B34" s="2">
         <v>5</v>
@@ -1810,7 +1829,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B35" s="2">
         <v>5</v>
@@ -1827,7 +1846,7 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="B36" s="2">
         <v>5</v>
@@ -1842,12 +1861,12 @@
         <v>156734</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="B37" s="2">
         <v>5</v>
@@ -1864,7 +1883,7 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="B38" s="2">
         <v>5</v>
@@ -1879,12 +1898,12 @@
         <v>59651</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="B39" s="2">
         <v>5</v>
@@ -1902,12 +1921,12 @@
         <v>16</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="B40" s="2">
         <v>5</v>
@@ -1919,12 +1938,12 @@
         <v>126903760</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="B41" s="2">
         <v>5</v>
@@ -1936,12 +1955,12 @@
         <v>126896451</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="B42" s="2">
         <v>5</v>
@@ -1962,11 +1981,915 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93210A17-976E-449D-A8F5-248F94CB6DA5}">
+  <dimension ref="A1:G42"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21.5703125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="6.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="104.85546875" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="3" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="2">
+        <v>5</v>
+      </c>
+      <c r="C2" s="2">
+        <v>126965629</v>
+      </c>
+      <c r="D2" s="2">
+        <v>126966115</v>
+      </c>
+      <c r="E2" s="2">
+        <v>277929</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="2">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2">
+        <v>126736375</v>
+      </c>
+      <c r="D3" s="2">
+        <v>126939807</v>
+      </c>
+      <c r="E3" s="2">
+        <v>203432</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="2">
+        <v>5</v>
+      </c>
+      <c r="C4" s="2">
+        <v>126742343</v>
+      </c>
+      <c r="D4" s="2">
+        <v>126932074</v>
+      </c>
+      <c r="E4" s="2">
+        <v>189731</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="2">
+        <v>5</v>
+      </c>
+      <c r="C5" s="2">
+        <v>126763901</v>
+      </c>
+      <c r="D5" s="2">
+        <v>126914184</v>
+      </c>
+      <c r="E5" s="2">
+        <v>150283</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="2">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2">
+        <v>126683194</v>
+      </c>
+      <c r="D6" s="2">
+        <v>126922135</v>
+      </c>
+      <c r="E6" s="2">
+        <v>238941</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="2">
+        <v>5</v>
+      </c>
+      <c r="C7" s="2">
+        <v>126761184</v>
+      </c>
+      <c r="D7" s="2">
+        <v>126930640</v>
+      </c>
+      <c r="E7" s="2">
+        <v>169456</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" s="2">
+        <v>5</v>
+      </c>
+      <c r="C8" s="2">
+        <v>126667591</v>
+      </c>
+      <c r="D8" s="2">
+        <v>127008376</v>
+      </c>
+      <c r="E8" s="2">
+        <v>340785</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="2">
+        <v>5</v>
+      </c>
+      <c r="C9" s="2">
+        <v>126705616</v>
+      </c>
+      <c r="D9" s="2">
+        <v>126909458</v>
+      </c>
+      <c r="E9" s="2">
+        <v>203842</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="2">
+        <v>5</v>
+      </c>
+      <c r="C10" s="2">
+        <v>126686881</v>
+      </c>
+      <c r="D10" s="2">
+        <v>126915553</v>
+      </c>
+      <c r="E10" s="2">
+        <v>228672</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" s="2">
+        <v>5</v>
+      </c>
+      <c r="C11" s="2">
+        <v>126766751</v>
+      </c>
+      <c r="D11" s="2">
+        <v>126995994</v>
+      </c>
+      <c r="E11" s="2">
+        <v>229243</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B12" s="2">
+        <v>5</v>
+      </c>
+      <c r="C12" s="2">
+        <v>126687731</v>
+      </c>
+      <c r="D12" s="2">
+        <v>126965660</v>
+      </c>
+      <c r="E12" s="2">
+        <v>277929</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" s="2">
+        <v>5</v>
+      </c>
+      <c r="C13" s="2">
+        <v>126775269</v>
+      </c>
+      <c r="D13" s="2">
+        <v>126893623</v>
+      </c>
+      <c r="E13" s="2">
+        <v>118354</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B14" s="2">
+        <v>5</v>
+      </c>
+      <c r="C14" s="2">
+        <v>126716573</v>
+      </c>
+      <c r="D14" s="2">
+        <v>126926882</v>
+      </c>
+      <c r="E14" s="2">
+        <v>210309</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B15" s="2">
+        <v>5</v>
+      </c>
+      <c r="C15" s="2">
+        <v>126743135</v>
+      </c>
+      <c r="D15" s="2">
+        <v>126865131</v>
+      </c>
+      <c r="E15" s="2">
+        <v>121996</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B16" s="2">
+        <v>5</v>
+      </c>
+      <c r="C16" s="2">
+        <v>125918128</v>
+      </c>
+      <c r="D16" s="2">
+        <v>126949480</v>
+      </c>
+      <c r="E16" s="2">
+        <v>1031351</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B17" s="2">
+        <v>5</v>
+      </c>
+      <c r="C17" s="2">
+        <v>126016772</v>
+      </c>
+      <c r="D17" s="2">
+        <v>126689287</v>
+      </c>
+      <c r="E17" s="2">
+        <v>672515</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B18" s="2">
+        <v>5</v>
+      </c>
+      <c r="C18" s="2">
+        <v>122477418</v>
+      </c>
+      <c r="D18" s="2">
+        <v>126843396</v>
+      </c>
+      <c r="E18" s="2">
+        <v>4365976</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B19" s="2">
+        <v>5</v>
+      </c>
+      <c r="C19" s="2">
+        <v>122477254</v>
+      </c>
+      <c r="D19" s="2">
+        <v>126843256</v>
+      </c>
+      <c r="E19" s="2">
+        <v>4366000</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B20" s="2">
+        <v>5</v>
+      </c>
+      <c r="C20" s="2">
+        <v>122476520</v>
+      </c>
+      <c r="D20" s="2">
+        <v>126842588</v>
+      </c>
+      <c r="E20" s="2">
+        <v>4366065</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B21" s="2">
+        <v>5</v>
+      </c>
+      <c r="C21" s="2">
+        <v>126050112</v>
+      </c>
+      <c r="D21" s="2">
+        <v>126707361</v>
+      </c>
+      <c r="E21" s="2">
+        <v>660000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B22" s="2">
+        <v>5</v>
+      </c>
+      <c r="C22" s="2">
+        <v>126156719</v>
+      </c>
+      <c r="D22" s="2">
+        <v>126765604</v>
+      </c>
+      <c r="E22" s="2">
+        <v>608833</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B23" s="2">
+        <v>5</v>
+      </c>
+      <c r="C23" s="2">
+        <v>126363827</v>
+      </c>
+      <c r="D23" s="2">
+        <v>126838825</v>
+      </c>
+      <c r="E23" s="2">
+        <v>474998</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B24" s="2">
+        <v>5</v>
+      </c>
+      <c r="C24" s="2">
+        <v>126512007</v>
+      </c>
+      <c r="D24" s="2">
+        <v>126978629</v>
+      </c>
+      <c r="E24" s="2">
+        <v>466623</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B25" s="2">
+        <v>5</v>
+      </c>
+      <c r="C25" s="2">
+        <v>126522203</v>
+      </c>
+      <c r="D25" s="2">
+        <v>126772687</v>
+      </c>
+      <c r="E25" s="2">
+        <v>250000</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="B26" s="2">
+        <v>5</v>
+      </c>
+      <c r="C26" s="2">
+        <v>126637847</v>
+      </c>
+      <c r="D26" s="2">
+        <v>126913193</v>
+      </c>
+      <c r="E26" s="2">
+        <v>275347</v>
+      </c>
+      <c r="G26" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B27" s="2">
+        <v>5</v>
+      </c>
+      <c r="C27" s="2">
+        <v>126695490</v>
+      </c>
+      <c r="D27" s="2">
+        <v>127036275</v>
+      </c>
+      <c r="E27" s="2">
+        <v>340785</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B28" s="2">
+        <v>5</v>
+      </c>
+      <c r="C28" s="2">
+        <v>126698430</v>
+      </c>
+      <c r="D28" s="2">
+        <v>126889630</v>
+      </c>
+      <c r="E28" s="2">
+        <v>191200</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G28" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B29" s="2">
+        <v>5</v>
+      </c>
+      <c r="C29" s="2">
+        <v>126705102</v>
+      </c>
+      <c r="D29" s="2">
+        <v>127029777</v>
+      </c>
+      <c r="E29" s="2">
+        <v>324675</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B30" s="2">
+        <v>5</v>
+      </c>
+      <c r="C30" s="2">
+        <v>126713540</v>
+      </c>
+      <c r="D30" s="2">
+        <v>126947560</v>
+      </c>
+      <c r="E30" s="2">
+        <v>234020</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B31" s="2">
+        <v>5</v>
+      </c>
+      <c r="C31" s="2">
+        <v>126718880</v>
+      </c>
+      <c r="D31" s="2">
+        <v>126866965</v>
+      </c>
+      <c r="E31" s="2">
+        <v>148085</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B32" s="2">
+        <v>5</v>
+      </c>
+      <c r="C32" s="2">
+        <v>126732318</v>
+      </c>
+      <c r="D32" s="2">
+        <v>126886087</v>
+      </c>
+      <c r="E32" s="2">
+        <v>153769</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B33" s="2">
+        <v>5</v>
+      </c>
+      <c r="C33" s="2">
+        <v>126736453</v>
+      </c>
+      <c r="D33" s="2">
+        <v>126864061</v>
+      </c>
+      <c r="E33" s="2">
+        <v>127608</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B34" s="2">
+        <v>5</v>
+      </c>
+      <c r="C34" s="2">
+        <v>126739243</v>
+      </c>
+      <c r="D34" s="2">
+        <v>127054568</v>
+      </c>
+      <c r="E34" s="2">
+        <v>315000</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B35" s="2">
+        <v>5</v>
+      </c>
+      <c r="C35" s="2">
+        <v>126763765</v>
+      </c>
+      <c r="D35" s="2">
+        <v>126913191</v>
+      </c>
+      <c r="E35" s="2">
+        <v>275540</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B36" s="2">
+        <v>5</v>
+      </c>
+      <c r="C36" s="2">
+        <v>126766199</v>
+      </c>
+      <c r="D36" s="2">
+        <v>126922932</v>
+      </c>
+      <c r="E36" s="2">
+        <v>156734</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B37" s="2">
+        <v>5</v>
+      </c>
+      <c r="C37" s="2">
+        <v>126762001</v>
+      </c>
+      <c r="D37" s="2">
+        <v>126997121</v>
+      </c>
+      <c r="E37" s="2">
+        <v>235000</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B38" s="2">
+        <v>5</v>
+      </c>
+      <c r="C38" s="2">
+        <v>126805047</v>
+      </c>
+      <c r="D38" s="2">
+        <v>126864688</v>
+      </c>
+      <c r="E38" s="2">
+        <v>59651</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B39" s="2">
+        <v>5</v>
+      </c>
+      <c r="C39" s="2">
+        <v>126729432</v>
+      </c>
+      <c r="D39" s="2">
+        <v>126915116</v>
+      </c>
+      <c r="E39" s="2">
+        <v>184808</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G39" s="5" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B40" s="2">
+        <v>5</v>
+      </c>
+      <c r="C40" s="2">
+        <v>126750808</v>
+      </c>
+      <c r="D40" s="2">
+        <v>126903760</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B41" s="2">
+        <v>5</v>
+      </c>
+      <c r="C41" s="2">
+        <v>126676886</v>
+      </c>
+      <c r="D41" s="2">
+        <v>126896451</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B42" s="2">
+        <v>5</v>
+      </c>
+      <c r="C42" s="2">
+        <v>126676469</v>
+      </c>
+      <c r="D42" s="2">
+        <v>126897351</v>
+      </c>
+      <c r="E42" s="2">
+        <v>221000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.42578125" style="2" customWidth="1"/>
     <col min="2" max="2" width="21.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" style="2" customWidth="1"/>
     <col min="4" max="4" width="14.7109375" style="2" customWidth="1"/>
@@ -2001,15 +2924,15 @@
         <v>16</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C3" s="2">
         <v>31</v>
@@ -2018,15 +2941,15 @@
         <v>45</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C4" s="2">
         <v>3</v>
@@ -2035,197 +2958,197 @@
         <v>43</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C5" s="2">
         <v>3</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="E7" s="5" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C9" s="2">
         <v>4</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C10" s="2">
         <v>4</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>75</v>
+        <v>214</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="C17" s="2">
         <v>3</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>81</v>
+        <v>215</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>82</v>
+        <v>216</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C19" s="2">
         <v>5</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>86</v>
+        <v>217</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C21" s="2">
         <v>32</v>
@@ -2233,10 +3156,10 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="C22" s="2">
         <v>1</v>
@@ -2245,37 +3168,37 @@
         <v>52</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>98</v>
+        <v>218</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="C25" s="2">
         <v>1</v>
@@ -2284,64 +3207,64 @@
         <v>34</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>106</v>
+        <v>219</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C31" s="2">
         <v>12</v>
@@ -2350,69 +3273,69 @@
         <v>45</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="C32" s="2">
         <v>8</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C38" s="2">
         <v>2</v>
@@ -2421,23 +3344,23 @@
         <v>58</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="C40" s="2">
         <v>6</v>
@@ -2446,41 +3369,41 @@
         <v>44</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="C41" s="2">
         <v>6</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="C42" s="2">
         <v>6</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -2488,12 +3411,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A753260-5018-4B3D-A2D6-F970E150F2D9}">
   <dimension ref="A1:E42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" style="2" customWidth="1"/>
     <col min="2" max="2" width="57.28515625" style="5" customWidth="1"/>
     <col min="3" max="3" width="105.42578125" style="5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.140625" style="2" customWidth="1"/>
@@ -2522,528 +3445,528 @@
         <v>15</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>19</v>
+        <v>213</v>
       </c>
       <c r="C2" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>20</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="D3" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B4" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="E4" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B6" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="D6" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="D7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="5" t="s">
         <v>54</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>50</v>
-      </c>
       <c r="D8" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>19</v>
       </c>
       <c r="C9" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="E9" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>19</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>50</v>
-      </c>
       <c r="D11" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>75</v>
+        <v>214</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>81</v>
+        <v>215</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>82</v>
+        <v>216</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>86</v>
+        <v>217</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B23" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C23" s="5" t="s">
-        <v>50</v>
-      </c>
       <c r="D23" s="2" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>98</v>
+        <v>218</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>106</v>
+        <v>219</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="B30" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C30" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C30" s="5" t="s">
-        <v>50</v>
-      </c>
       <c r="D30" s="2" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>175</v>
-      </c>
-      <c r="B40" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="D41" s="2" t="s">
         <v>176</v>
-      </c>
-      <c r="B41" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="C41" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corrected spelling of summary
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\Krizchelle\ADLD Patient Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2388684B-CA99-4C5B-AD67-D7724DF1017F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A03D514F-A297-44FB-B3EA-CD2554FF70A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -701,9 +701,6 @@
     <t>NonADLD_dup_6</t>
   </si>
   <si>
-    <t>Summarry</t>
-  </si>
-  <si>
     <t>Testing 1</t>
   </si>
   <si>
@@ -825,6 +822,9 @@
   </si>
   <si>
     <t>Testing 41</t>
+  </si>
+  <si>
+    <t>Summary</t>
   </si>
 </sst>
 </file>
@@ -2106,12 +2106,12 @@
     <col min="2" max="2" width="95.7109375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>220</v>
+        <v>261</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -2119,7 +2119,7 @@
         <v>15</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -2127,7 +2127,7 @@
         <v>22</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -2135,7 +2135,7 @@
         <v>29</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -2143,7 +2143,7 @@
         <v>30</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -2151,7 +2151,7 @@
         <v>31</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -2159,7 +2159,7 @@
         <v>32</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -2167,7 +2167,7 @@
         <v>55</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -2175,7 +2175,7 @@
         <v>56</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -2183,7 +2183,7 @@
         <v>57</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -2191,7 +2191,7 @@
         <v>58</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -2199,7 +2199,7 @@
         <v>69</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -2207,7 +2207,7 @@
         <v>70</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -2215,7 +2215,7 @@
         <v>71</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -2223,7 +2223,7 @@
         <v>73</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -2231,7 +2231,7 @@
         <v>214</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -2239,7 +2239,7 @@
         <v>75</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -2247,7 +2247,7 @@
         <v>215</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -2255,7 +2255,7 @@
         <v>216</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -2263,7 +2263,7 @@
         <v>217</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -2271,7 +2271,7 @@
         <v>82</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -2279,7 +2279,7 @@
         <v>83</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -2287,7 +2287,7 @@
         <v>88</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -2295,7 +2295,7 @@
         <v>218</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -2303,7 +2303,7 @@
         <v>99</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -2311,7 +2311,7 @@
         <v>219</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -2319,7 +2319,7 @@
         <v>120</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -2327,7 +2327,7 @@
         <v>101</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -2335,7 +2335,7 @@
         <v>103</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -2343,7 +2343,7 @@
         <v>105</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -2351,7 +2351,7 @@
         <v>107</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
@@ -2359,7 +2359,7 @@
         <v>109</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -2367,7 +2367,7 @@
         <v>121</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
@@ -2375,7 +2375,7 @@
         <v>122</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
@@ -2383,7 +2383,7 @@
         <v>124</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
@@ -2391,7 +2391,7 @@
         <v>142</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
@@ -2399,7 +2399,7 @@
         <v>125</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
@@ -2407,7 +2407,7 @@
         <v>126</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -2415,7 +2415,7 @@
         <v>143</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
@@ -2423,7 +2423,7 @@
         <v>168</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
@@ -2431,7 +2431,7 @@
         <v>169</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -2439,7 +2439,7 @@
         <v>193</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel sheet to test the line break
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\Krizchelle\ADLD Patient Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A03D514F-A297-44FB-B3EA-CD2554FF70A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B10F53F7-6FDF-43AB-8BE8-BC025BE52818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -710,9 +710,6 @@
     <t>Testing 3</t>
   </si>
   <si>
-    <t>Testing 4</t>
-  </si>
-  <si>
     <t>Testing 5</t>
   </si>
   <si>
@@ -825,6 +822,10 @@
   </si>
   <si>
     <t>Summary</t>
+  </si>
+  <si>
+    <t>Testing 4
+Testing for line break 4</t>
   </si>
 </sst>
 </file>
@@ -894,7 +895,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -913,6 +914,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2111,7 +2115,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -2138,12 +2142,12 @@
         <v>222</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>223</v>
+      <c r="B5" s="7" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -2151,7 +2155,7 @@
         <v>31</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -2159,7 +2163,7 @@
         <v>32</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -2167,7 +2171,7 @@
         <v>55</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -2175,7 +2179,7 @@
         <v>56</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -2183,7 +2187,7 @@
         <v>57</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -2191,7 +2195,7 @@
         <v>58</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -2199,7 +2203,7 @@
         <v>69</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -2207,7 +2211,7 @@
         <v>70</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -2215,7 +2219,7 @@
         <v>71</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -2223,7 +2227,7 @@
         <v>73</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -2231,7 +2235,7 @@
         <v>214</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -2239,7 +2243,7 @@
         <v>75</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -2247,7 +2251,7 @@
         <v>215</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -2255,7 +2259,7 @@
         <v>216</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -2263,7 +2267,7 @@
         <v>217</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -2271,7 +2275,7 @@
         <v>82</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -2279,7 +2283,7 @@
         <v>83</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -2287,7 +2291,7 @@
         <v>88</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -2295,7 +2299,7 @@
         <v>218</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -2303,7 +2307,7 @@
         <v>99</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -2311,7 +2315,7 @@
         <v>219</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -2319,7 +2323,7 @@
         <v>120</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -2327,7 +2331,7 @@
         <v>101</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -2335,7 +2339,7 @@
         <v>103</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -2343,7 +2347,7 @@
         <v>105</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -2351,7 +2355,7 @@
         <v>107</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
@@ -2359,7 +2363,7 @@
         <v>109</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -2367,7 +2371,7 @@
         <v>121</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
@@ -2375,7 +2379,7 @@
         <v>122</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
@@ -2383,7 +2387,7 @@
         <v>124</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
@@ -2391,7 +2395,7 @@
         <v>142</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
@@ -2399,7 +2403,7 @@
         <v>125</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
@@ -2407,7 +2411,7 @@
         <v>126</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -2415,7 +2419,7 @@
         <v>143</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
@@ -2423,7 +2427,7 @@
         <v>168</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
@@ -2431,7 +2435,7 @@
         <v>169</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -2439,7 +2443,7 @@
         <v>193</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added template for evidence summary section
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\Krizchelle\ADLD Patient Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B10F53F7-6FDF-43AB-8BE8-BC025BE52818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{291A3522-770D-4749-80B3-7132C0919991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Molecular" sheetId="4" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="222">
   <si>
     <t>Item name</t>
   </si>
@@ -701,131 +701,15 @@
     <t>NonADLD_dup_6</t>
   </si>
   <si>
-    <t>Testing 1</t>
-  </si>
-  <si>
-    <t>Testing 2</t>
-  </si>
-  <si>
-    <t>Testing 3</t>
-  </si>
-  <si>
-    <t>Testing 5</t>
-  </si>
-  <si>
-    <t>Testing 6</t>
-  </si>
-  <si>
-    <t>Testing 7</t>
-  </si>
-  <si>
-    <t>Testing 8</t>
-  </si>
-  <si>
-    <t>Testing 9</t>
-  </si>
-  <si>
-    <t>Testing 10</t>
-  </si>
-  <si>
-    <t>Testing 11</t>
-  </si>
-  <si>
-    <t>Testing 12</t>
-  </si>
-  <si>
-    <t>Testing 13</t>
-  </si>
-  <si>
-    <t>Testing 14</t>
-  </si>
-  <si>
-    <t>Testing 15</t>
-  </si>
-  <si>
-    <t>Testing 16</t>
-  </si>
-  <si>
-    <t>Testing 17</t>
-  </si>
-  <si>
-    <t>Testing 18</t>
-  </si>
-  <si>
-    <t>Testing 19</t>
-  </si>
-  <si>
-    <t>Testing 20</t>
-  </si>
-  <si>
-    <t>Testing 21</t>
-  </si>
-  <si>
-    <t>Testing 22</t>
-  </si>
-  <si>
-    <t>Testing 23</t>
-  </si>
-  <si>
-    <t>Testing 24</t>
-  </si>
-  <si>
-    <t>Testing 25</t>
-  </si>
-  <si>
-    <t>Testing 26</t>
-  </si>
-  <si>
-    <t>Testing 27</t>
-  </si>
-  <si>
-    <t>Testing 28</t>
-  </si>
-  <si>
-    <t>Testing 29</t>
-  </si>
-  <si>
-    <t>Testing 30</t>
-  </si>
-  <si>
-    <t>Testing 31</t>
-  </si>
-  <si>
-    <t>Testing 32</t>
-  </si>
-  <si>
-    <t>Testing 33</t>
-  </si>
-  <si>
-    <t>Testing 34</t>
-  </si>
-  <si>
-    <t>Testing 35</t>
-  </si>
-  <si>
-    <t>Testing 36</t>
-  </si>
-  <si>
-    <t>Testing 37</t>
-  </si>
-  <si>
-    <t>Testing 38</t>
-  </si>
-  <si>
-    <t>Testing 39</t>
-  </si>
-  <si>
-    <t>Testing 40</t>
-  </si>
-  <si>
-    <t>Testing 41</t>
-  </si>
-  <si>
     <t>Summary</t>
   </si>
   <si>
-    <t>Testing 4
-Testing for line break 4</t>
+    <t xml:space="preserve">publications
+literature case labels
+multigenerational family
+estimated unique individuals
+high-confidence linked individuals
+Deduplication status: </t>
   </si>
 </sst>
 </file>
@@ -2115,335 +1999,335 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B2" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B3" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="B4" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B6" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B7" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B8" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B9" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B10" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B11" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B12" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B13" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B14" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B15" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B16" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B17" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B18" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B19" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B20" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B21" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B22" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B23" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B24" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B25" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B26" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B27" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B28" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B29" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B30" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B31" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B32" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B33" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B34" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B35" s="2" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B35" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B36" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B37" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="B38" s="2" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B38" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B39" s="2" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B39" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="B40" s="2" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B40" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B41" s="2" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B41" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="B42" s="2" t="s">
-        <v>259</v>
+      <c r="B42" s="7" t="s">
+        <v>221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deleted duplication found in symptoms sheet
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\Krizchelle\ADLD Patient Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4714D92F-4B78-40C2-AED9-46CFA1B8DF30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D46D060-F624-485D-94EE-A02F6AE57953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Molecular" sheetId="4" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="227">
   <si>
     <t>Item name</t>
   </si>
@@ -83,15 +83,6 @@
     <t>Canada</t>
   </si>
   <si>
-    <t>10.1002/humu.22348, 10.1007/s10048-010-0269-y</t>
-  </si>
-  <si>
-    <t>10.1001/archneur.65.11.1496</t>
-  </si>
-  <si>
-    <t>A1, CA2</t>
-  </si>
-  <si>
     <t>ADLD_dup_2</t>
   </si>
   <si>
@@ -101,18 +92,6 @@
     <t>Sweden</t>
   </si>
   <si>
-    <t>10.1002/humu.22348, 10.1007/s10048-010-0269-y, PMC8133955, 10.3174/ajnr.A1354, 10.1002/ajmg.b.30342, 10.1002/ana.24452</t>
-  </si>
-  <si>
-    <t>Giorgio 2013, Schuster 2011, Melberg 2006, Sundbloom 2008, Marklund 2006, Finnsson 2015</t>
-  </si>
-  <si>
-    <t>SE1, A2</t>
-  </si>
-  <si>
-    <t>10.1007/s10048-010-0269-y</t>
-  </si>
-  <si>
     <t>ADLD_dup_3</t>
   </si>
   <si>
@@ -146,45 +125,9 @@
     <t>40.5 ± 4.9</t>
   </si>
   <si>
-    <t>10.1002/humu.22348, 10.1007/s10048-010-0269-y, PMC8133955, 10.3174/ajnr.A1354, 10.1002/ana.24452</t>
-  </si>
-  <si>
-    <t>Giorgio 2013, Schuster 2011, Melberg 2006, Sundbloom 2008, Finnsson 2015</t>
-  </si>
-  <si>
-    <t>SE2, A3</t>
-  </si>
-  <si>
-    <t>10.1002/humu.22348, 10.1002/mds.24064</t>
-  </si>
-  <si>
-    <t>Giorgio 2013, Fogel 2012</t>
-  </si>
-  <si>
-    <t>A4</t>
-  </si>
-  <si>
-    <t>10.1002/humu.22348</t>
-  </si>
-  <si>
     <t>Giorgio 2013</t>
   </si>
   <si>
-    <t>A5</t>
-  </si>
-  <si>
-    <t>10.1002/humu.22348, 10.1038/ng1872, https://doi.org/10.1093/hmg/9.5.787</t>
-  </si>
-  <si>
-    <t>Giorgio 2013, Padiath 2006, Coffeen 2000</t>
-  </si>
-  <si>
-    <t>A6, A7, K2-3, K2685, K50069</t>
-  </si>
-  <si>
-    <t>10.1038/ng1872</t>
-  </si>
-  <si>
     <t>ADLD_dup_7</t>
   </si>
   <si>
@@ -209,21 +152,6 @@
     <t>53, 58</t>
   </si>
   <si>
-    <t>A8, AV1</t>
-  </si>
-  <si>
-    <t>Giorgio 2013, Schuster 2011</t>
-  </si>
-  <si>
-    <t>IL, A10</t>
-  </si>
-  <si>
-    <t>DE, A11</t>
-  </si>
-  <si>
-    <t>A14</t>
-  </si>
-  <si>
     <t>Microhomology of "GG"</t>
   </si>
   <si>
@@ -251,18 +179,6 @@
     <t>Nmezi 2019</t>
   </si>
   <si>
-    <t>DEL3-1, DEL3-2, DEL3-3</t>
-  </si>
-  <si>
-    <t>10.1212/NXG.0000000000000305</t>
-  </si>
-  <si>
-    <t>Nmezi et al. 2025</t>
-  </si>
-  <si>
-    <t>10.1038/s41467-025-56378-9</t>
-  </si>
-  <si>
     <t>Britain, England</t>
   </si>
   <si>
@@ -272,18 +188,6 @@
     <t>ADLD_del_3</t>
   </si>
   <si>
-    <t>Quattrocolo et al. 1997, Brussino et al. 2010, Giorgio et al. 2015, Giordana et al. 2005, Piccinini et al. 2009</t>
-  </si>
-  <si>
-    <t>ADLD-1-TO</t>
-  </si>
-  <si>
-    <t>Nmezi 2019, Alturkustani 2013</t>
-  </si>
-  <si>
-    <t>CA-Del; CA2; S4; 1_3; DEL2-1, AC-11-519(Deletion)</t>
-  </si>
-  <si>
     <t>ADLD_invdup_1</t>
   </si>
   <si>
@@ -296,27 +200,12 @@
     <t>Brazil</t>
   </si>
   <si>
-    <t>BR1</t>
-  </si>
-  <si>
-    <t>10.1212/NXG.0000000000200261</t>
-  </si>
-  <si>
     <t>Wang 2025</t>
   </si>
   <si>
     <t>Alujr centromeric repeat, AluSP telomeric repeat, no microhomology at junctions</t>
   </si>
   <si>
-    <t>10.1002/humu.22348, 10.1001/archneur.65.11.1496, https://doi.org/10.1212/NXG.0000000000000305, 10.1097/NEN.0000000000000008</t>
-  </si>
-  <si>
-    <t>Giorgio, et al. 2013, Meijer et al. 2008, Nmezi et al. 2019, Alturkustani et al. 2013</t>
-  </si>
-  <si>
-    <t>DEL1-1</t>
-  </si>
-  <si>
     <t>ADLD_del_4</t>
   </si>
   <si>
@@ -356,30 +245,6 @@
     <t>France</t>
   </si>
   <si>
-    <t>10.1038/ng1873, PMID: 8958750</t>
-  </si>
-  <si>
-    <t>Padiath 2006, Asahara 1996</t>
-  </si>
-  <si>
-    <t>K50069</t>
-  </si>
-  <si>
-    <t>10.1002/humu.22348, 10.1016/j.autneu.2010.07.011</t>
-  </si>
-  <si>
-    <t>FR1, FR2</t>
-  </si>
-  <si>
-    <t>10.1002/humu.22348, 10.1007/s00415-011-6225-4</t>
-  </si>
-  <si>
-    <t>Giorgio 2013, Dos Santos 2011</t>
-  </si>
-  <si>
-    <t>10.1007/s00415-011-6225-4</t>
-  </si>
-  <si>
     <t>ADLD_dup_15</t>
   </si>
   <si>
@@ -416,36 +281,6 @@
     <t>Uruguay</t>
   </si>
   <si>
-    <t>10.1002/humu.22348, 10.1111/j.1468-1331.2009.02536.x</t>
-  </si>
-  <si>
-    <t>Giorgio 2013, Brussino 2008</t>
-  </si>
-  <si>
-    <t>IT1</t>
-  </si>
-  <si>
-    <t>10.1111/j.1468-1331.2009.02536.x</t>
-  </si>
-  <si>
-    <t>IT2</t>
-  </si>
-  <si>
-    <t>10.1016/j.bbadis.2012.12.006 10.1093/hmg/ddv034</t>
-  </si>
-  <si>
-    <t>Columbaro et al. 2013, Barlotelli-Stella et al. 2015</t>
-  </si>
-  <si>
-    <t>ADLD2</t>
-  </si>
-  <si>
-    <t>10.3389/fnins.2019.01030</t>
-  </si>
-  <si>
-    <t>1_3</t>
-  </si>
-  <si>
     <t>ADLD_dup_24</t>
   </si>
   <si>
@@ -455,12 +290,6 @@
     <t>220 kb</t>
   </si>
   <si>
-    <t>10.1212/nxg.0000000000000292</t>
-  </si>
-  <si>
-    <t>Mezaki et al. 2018</t>
-  </si>
-  <si>
     <t>N/A</t>
   </si>
   <si>
@@ -503,15 +332,6 @@
     <t>Microhomology of "AA"</t>
   </si>
   <si>
-    <t>10.1212/NXG.0000000000000305, 10.1097/NEN.0000000000000008</t>
-  </si>
-  <si>
-    <t>10.1159/000117406, 10.1111/j.1468-1331.2009.02844.x, 10.1093/hmg/ddv065, 10.1111/j.1750-3639.2005.tb00506.x, 10.1111/j.1750-3639.2009.00313.x</t>
-  </si>
-  <si>
-    <t>10.1111/j.1468-1331.2009.02844.x, 10.1093/hmg/ddv065</t>
-  </si>
-  <si>
     <t>ADLD_dup_28</t>
   </si>
   <si>
@@ -533,24 +353,9 @@
     <t>55, 52, 50</t>
   </si>
   <si>
-    <t>Pedigree I - Patient I</t>
-  </si>
-  <si>
-    <t>Pedigree II - Patient 2, Pedigree II - Patient 3, Pedigree III - Patient 4</t>
-  </si>
-  <si>
-    <t>F2-1, F2-2, F2-3</t>
-  </si>
-  <si>
-    <t>F1, F1-1, F1-2, F1-3, F1-4, F1-5, GM B206</t>
-  </si>
-  <si>
     <t>Northern European</t>
   </si>
   <si>
-    <t>F3-1, F3-2</t>
-  </si>
-  <si>
     <t>Southern Italy</t>
   </si>
   <si>
@@ -560,40 +365,16 @@
     <t>48, 50, 48, 42</t>
   </si>
   <si>
-    <t>Giorgio 2013, Guaraldi 2011, Terlizzi et al. 2016</t>
-  </si>
-  <si>
-    <t>IT3, IV11, IV10, IV12</t>
-  </si>
-  <si>
-    <t>10.1038/ng1872, 10.1016/j.autneu/2016.02.005</t>
-  </si>
-  <si>
-    <t>Zhang et al. 2019</t>
-  </si>
-  <si>
-    <t>Proband II-4</t>
-  </si>
-  <si>
     <t>China</t>
   </si>
   <si>
     <t>Predicted junction</t>
   </si>
   <si>
-    <t>GR1</t>
-  </si>
-  <si>
     <t>Korea</t>
   </si>
   <si>
     <t>ADLD_dup_30</t>
-  </si>
-  <si>
-    <t>Pedigree III - Patient 4</t>
-  </si>
-  <si>
-    <t>10.1002/humu.22348, 10.1007/s10048-010-0269-y, 10.1001/archneur.65.11.1496</t>
   </si>
   <si>
     <t>NonADLD_dup_1</t>
@@ -643,12 +424,6 @@
     <t>Cases reported</t>
   </si>
   <si>
-    <t>Giorgio 2013, Schuster 2011, Meijer 2008 *pedigree TEST</t>
-  </si>
-  <si>
-    <t>Giorgio 2013, Schuster 2011, Meijer 2008 TEST</t>
-  </si>
-  <si>
     <t>[Symptomatic - specific symptoms not documented] [Autonomic dysfunction] [Orthostatic hypotension] [Bladder/bowel dysfunction] [Sexual dysfunction] [Thermoregulatory dysfunction] [Pyramidal signs]</t>
   </si>
   <si>
@@ -828,9 +603,6 @@
     <t>Meijer2008_IV1; _II3; _II4; _III10; _IV13; _IV4</t>
   </si>
   <si>
-    <t>Meijer_2008</t>
-  </si>
-  <si>
     <t>Marklund2008_Cohort</t>
   </si>
   <si>
@@ -952,6 +724,9 @@
   </si>
   <si>
     <t>Zhang2019_II4_Proband; Zhang2019_II5</t>
+  </si>
+  <si>
+    <t>Meijer 2008</t>
   </si>
 </sst>
 </file>
@@ -1402,7 +1177,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B3" s="2">
         <v>5</v>
@@ -1420,12 +1195,12 @@
         <v>11</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B4" s="2">
         <v>5</v>
@@ -1443,12 +1218,12 @@
         <v>11</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>146</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B5" s="2">
         <v>5</v>
@@ -1466,12 +1241,12 @@
         <v>11</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>145</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B6" s="2">
         <v>5</v>
@@ -1489,12 +1264,12 @@
         <v>11</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>144</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B7" s="2">
         <v>5</v>
@@ -1509,15 +1284,15 @@
         <v>169456</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="B8" s="2">
         <v>5</v>
@@ -1532,15 +1307,15 @@
         <v>340785</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>147</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="B9" s="2">
         <v>5</v>
@@ -1558,12 +1333,12 @@
         <v>11</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>148</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="B10" s="2">
         <v>5</v>
@@ -1581,12 +1356,12 @@
         <v>11</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>61</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="B11" s="2">
         <v>5</v>
@@ -1604,12 +1379,12 @@
         <v>11</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>149</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="B12" s="2">
         <v>5</v>
@@ -1626,7 +1401,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="B13" s="2">
         <v>5</v>
@@ -1644,12 +1419,12 @@
         <v>11</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>143</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="B14" s="2">
         <v>5</v>
@@ -1667,12 +1442,12 @@
         <v>11</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>65</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>66</v>
+        <v>42</v>
       </c>
       <c r="B15" s="2">
         <v>5</v>
@@ -1689,7 +1464,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>185</v>
+        <v>112</v>
       </c>
       <c r="B16" s="2">
         <v>5</v>
@@ -1707,12 +1482,12 @@
         <v>11</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>141</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="B17" s="2">
         <v>5</v>
@@ -1727,15 +1502,15 @@
         <v>672515</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>140</v>
+        <v>83</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>142</v>
+        <v>85</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>186</v>
+        <v>113</v>
       </c>
       <c r="B18" s="2">
         <v>5</v>
@@ -1750,12 +1525,12 @@
         <v>4365976</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>150</v>
+        <v>93</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>187</v>
+        <v>114</v>
       </c>
       <c r="B19" s="2">
         <v>5</v>
@@ -1770,12 +1545,12 @@
         <v>4366000</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>151</v>
+        <v>94</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>188</v>
+        <v>115</v>
       </c>
       <c r="B20" s="2">
         <v>5</v>
@@ -1792,7 +1567,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="B21" s="2">
         <v>5</v>
@@ -1809,7 +1584,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="B22" s="2">
         <v>5</v>
@@ -1824,15 +1599,15 @@
         <v>608833</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>140</v>
+        <v>83</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>152</v>
+        <v>95</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>81</v>
+        <v>49</v>
       </c>
       <c r="B23" s="2">
         <v>5</v>
@@ -1847,15 +1622,15 @@
         <v>474998</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>82</v>
+        <v>50</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>83</v>
+        <v>51</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>189</v>
+        <v>116</v>
       </c>
       <c r="B24" s="2">
         <v>5</v>
@@ -1872,7 +1647,7 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>92</v>
+        <v>55</v>
       </c>
       <c r="B25" s="2">
         <v>5</v>
@@ -1887,15 +1662,15 @@
         <v>250000</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>140</v>
+        <v>83</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>88</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>190</v>
+        <v>117</v>
       </c>
       <c r="B26" s="2">
         <v>5</v>
@@ -1910,12 +1685,12 @@
         <v>275347</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>93</v>
+        <v>56</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>113</v>
+        <v>68</v>
       </c>
       <c r="B27" s="2">
         <v>5</v>
@@ -1933,12 +1708,12 @@
         <v>11</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>95</v>
+        <v>58</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>94</v>
+        <v>57</v>
       </c>
       <c r="B28" s="2">
         <v>5</v>
@@ -1956,12 +1731,12 @@
         <v>11</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>97</v>
+        <v>60</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>96</v>
+        <v>59</v>
       </c>
       <c r="B29" s="2">
         <v>5</v>
@@ -1979,12 +1754,12 @@
         <v>11</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>99</v>
+        <v>62</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>98</v>
+        <v>61</v>
       </c>
       <c r="B30" s="2">
         <v>5</v>
@@ -2002,12 +1777,12 @@
         <v>11</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>101</v>
+        <v>64</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="B31" s="2">
         <v>5</v>
@@ -2025,12 +1800,12 @@
         <v>11</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>103</v>
+        <v>66</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>102</v>
+        <v>65</v>
       </c>
       <c r="B32" s="2">
         <v>5</v>
@@ -2048,12 +1823,12 @@
         <v>11</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>153</v>
+        <v>96</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>114</v>
+        <v>69</v>
       </c>
       <c r="B33" s="2">
         <v>5</v>
@@ -2071,12 +1846,12 @@
         <v>11</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>116</v>
+        <v>71</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>115</v>
+        <v>70</v>
       </c>
       <c r="B34" s="2">
         <v>5</v>
@@ -2093,7 +1868,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>117</v>
+        <v>72</v>
       </c>
       <c r="B35" s="2">
         <v>5</v>
@@ -2110,7 +1885,7 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>135</v>
+        <v>80</v>
       </c>
       <c r="B36" s="2">
         <v>5</v>
@@ -2125,12 +1900,12 @@
         <v>156734</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>120</v>
+        <v>75</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>118</v>
+        <v>73</v>
       </c>
       <c r="B37" s="2">
         <v>5</v>
@@ -2147,7 +1922,7 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>119</v>
+        <v>74</v>
       </c>
       <c r="B38" s="2">
         <v>5</v>
@@ -2162,12 +1937,12 @@
         <v>59651</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>179</v>
+        <v>109</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>136</v>
+        <v>81</v>
       </c>
       <c r="B39" s="2">
         <v>5</v>
@@ -2185,12 +1960,12 @@
         <v>11</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>121</v>
+        <v>76</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>157</v>
+        <v>97</v>
       </c>
       <c r="B40" s="2">
         <v>5</v>
@@ -2202,12 +1977,12 @@
         <v>126903760</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>137</v>
+        <v>82</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>158</v>
+        <v>98</v>
       </c>
       <c r="B41" s="2">
         <v>5</v>
@@ -2219,12 +1994,12 @@
         <v>126896451</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>137</v>
+        <v>82</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>182</v>
+        <v>111</v>
       </c>
       <c r="B42" s="2">
         <v>5</v>
@@ -2258,7 +2033,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>191</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2266,327 +2041,327 @@
         <v>10</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>66</v>
+        <v>42</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>185</v>
+        <v>112</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>186</v>
+        <v>113</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>187</v>
+        <v>114</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>188</v>
+        <v>115</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>81</v>
+        <v>49</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>189</v>
+        <v>116</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>92</v>
+        <v>55</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>190</v>
+        <v>117</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>113</v>
+        <v>68</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>94</v>
+        <v>57</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>96</v>
+        <v>59</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>98</v>
+        <v>61</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>102</v>
+        <v>65</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>114</v>
+        <v>69</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>115</v>
+        <v>70</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>117</v>
+        <v>72</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>135</v>
+        <v>80</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>118</v>
+        <v>73</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>119</v>
+        <v>74</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>136</v>
+        <v>81</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>157</v>
+        <v>97</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>158</v>
+        <v>98</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>182</v>
+        <v>111</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>192</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -2613,7 +2388,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>193</v>
+        <v>120</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>7</v>
@@ -2622,10 +2397,10 @@
         <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>194</v>
+        <v>121</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>195</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2639,18 +2414,18 @@
         <v>16</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>201</v>
+        <v>126</v>
       </c>
       <c r="F2" t="s">
-        <v>202</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C3" s="2">
         <v>31</v>
@@ -2659,18 +2434,18 @@
         <v>45</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>203</v>
+        <v>128</v>
       </c>
       <c r="F3" t="s">
-        <v>204</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C4" s="2">
         <v>3</v>
@@ -2679,217 +2454,217 @@
         <v>43</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>205</v>
+        <v>130</v>
       </c>
       <c r="F4" t="s">
-        <v>206</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C5" s="2">
         <v>3</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>208</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>208</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>34</v>
-      </c>
       <c r="E7" s="5" t="s">
-        <v>210</v>
+        <v>135</v>
       </c>
       <c r="F7" t="s">
-        <v>211</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>208</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="C9" s="2">
         <v>4</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>208</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="C10" s="2">
         <v>4</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>208</v>
+        <v>133</v>
       </c>
       <c r="F10" t="s">
-        <v>215</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>208</v>
+        <v>133</v>
       </c>
       <c r="F11" t="s">
-        <v>215</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>62</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>63</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>64</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>66</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>185</v>
+        <v>112</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>67</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>160</v>
+        <v>100</v>
       </c>
       <c r="C17" s="2">
         <v>3</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>161</v>
+        <v>101</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>217</v>
+        <v>142</v>
       </c>
       <c r="F17" t="s">
-        <v>218</v>
+        <v>143</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>186</v>
+        <v>113</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>187</v>
+        <v>114</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>74</v>
+        <v>46</v>
       </c>
       <c r="C19" s="2">
         <v>5</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>219</v>
+        <v>144</v>
       </c>
       <c r="F19" t="s">
-        <v>220</v>
+        <v>145</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>188</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="C21" s="2">
         <v>32</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>221</v>
+        <v>146</v>
       </c>
       <c r="F21" t="s">
-        <v>222</v>
+        <v>147</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>162</v>
+        <v>102</v>
       </c>
       <c r="C22" s="2">
         <v>1</v>
@@ -2898,43 +2673,43 @@
         <v>52</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>223</v>
+        <v>148</v>
       </c>
       <c r="F22" t="s">
-        <v>218</v>
+        <v>143</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>81</v>
+        <v>49</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>84</v>
+        <v>52</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>205</v>
+        <v>130</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>189</v>
+        <v>116</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>168</v>
+        <v>104</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>224</v>
+        <v>149</v>
       </c>
       <c r="F24" t="s">
-        <v>220</v>
+        <v>145</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>92</v>
+        <v>55</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>181</v>
+        <v>110</v>
       </c>
       <c r="C25" s="2">
         <v>1</v>
@@ -2943,73 +2718,73 @@
         <v>34</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>225</v>
+        <v>150</v>
       </c>
       <c r="F25" t="s">
-        <v>226</v>
+        <v>151</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>190</v>
+        <v>117</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>228</v>
+        <v>153</v>
       </c>
       <c r="F26" t="s">
-        <v>229</v>
+        <v>154</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>113</v>
+        <v>68</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>208</v>
+        <v>133</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>94</v>
+        <v>57</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>96</v>
+        <v>59</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>170</v>
+        <v>105</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>171</v>
+        <v>106</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>172</v>
+        <v>107</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>231</v>
+        <v>156</v>
       </c>
       <c r="F29" t="s">
-        <v>232</v>
+        <v>157</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>98</v>
+        <v>61</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>104</v>
+        <v>67</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>208</v>
+        <v>133</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="C31" s="2">
         <v>12</v>
@@ -3018,75 +2793,75 @@
         <v>45</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>234</v>
+        <v>159</v>
       </c>
       <c r="F31" t="s">
-        <v>235</v>
+        <v>160</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>102</v>
+        <v>65</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>122</v>
+        <v>77</v>
       </c>
       <c r="C32" s="2">
         <v>8</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>123</v>
+        <v>78</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>208</v>
+        <v>133</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>114</v>
+        <v>69</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>208</v>
+        <v>133</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>115</v>
+        <v>70</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>238</v>
+        <v>163</v>
       </c>
       <c r="F34" t="s">
-        <v>239</v>
+        <v>164</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>117</v>
+        <v>72</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>135</v>
+        <v>80</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>118</v>
+        <v>73</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>241</v>
+        <v>166</v>
       </c>
       <c r="F37" t="s">
-        <v>239</v>
+        <v>164</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>119</v>
+        <v>74</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>178</v>
+        <v>108</v>
       </c>
       <c r="C38" s="2">
         <v>2</v>
@@ -3095,26 +2870,26 @@
         <v>58</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>242</v>
+        <v>167</v>
       </c>
       <c r="F38" t="s">
-        <v>243</v>
+        <v>168</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>136</v>
+        <v>81</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>124</v>
+        <v>79</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>157</v>
+        <v>97</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>159</v>
+        <v>99</v>
       </c>
       <c r="C40" s="2">
         <v>6</v>
@@ -3123,50 +2898,50 @@
         <v>44</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>245</v>
+        <v>170</v>
       </c>
       <c r="F40" t="s">
-        <v>226</v>
+        <v>151</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>158</v>
+        <v>98</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>159</v>
+        <v>99</v>
       </c>
       <c r="C41" s="2">
         <v>6</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>163</v>
+        <v>103</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>247</v>
+        <v>172</v>
       </c>
       <c r="F41" t="s">
-        <v>226</v>
+        <v>151</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>182</v>
+        <v>111</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>159</v>
+        <v>99</v>
       </c>
       <c r="C42" s="2">
         <v>6</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>163</v>
+        <v>103</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>249</v>
+        <v>174</v>
       </c>
       <c r="F42" t="s">
-        <v>226</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -3176,7 +2951,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A753260-5018-4B3D-A2D6-F970E150F2D9}">
-  <dimension ref="A1:F124"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="2" customWidth="1"/>
@@ -3191,13 +2966,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>197</v>
+        <v>124</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>196</v>
+        <v>123</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>198</v>
+        <v>125</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>9</v>
@@ -3208,13 +2983,13 @@
         <v>10</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C2" s="2">
         <v>23649844</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>258</v>
+        <v>183</v>
       </c>
       <c r="E2"/>
     </row>
@@ -3223,97 +2998,97 @@
         <v>10</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>260</v>
+        <v>226</v>
       </c>
       <c r="C3" s="2">
         <v>19001169</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>259</v>
+        <v>184</v>
       </c>
       <c r="E3"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>250</v>
+        <v>175</v>
       </c>
       <c r="C4" s="2">
         <v>16823806</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>261</v>
+        <v>185</v>
       </c>
       <c r="E4"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>266</v>
+        <v>190</v>
       </c>
       <c r="C5" s="2">
         <v>26053668</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>262</v>
+        <v>186</v>
       </c>
       <c r="E5"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C6" s="2">
         <v>23649844</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>263</v>
+        <v>187</v>
       </c>
       <c r="E6"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>267</v>
+        <v>191</v>
       </c>
       <c r="C7" s="2">
         <v>18945794</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>264</v>
+        <v>188</v>
       </c>
       <c r="E7"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>268</v>
+        <v>192</v>
       </c>
       <c r="C8" s="2">
         <v>24128683</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>265</v>
+        <v>189</v>
       </c>
       <c r="E8"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>266</v>
+        <v>190</v>
       </c>
       <c r="C9" s="2">
         <v>26053668</v>
@@ -3323,202 +3098,202 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C10" s="2">
         <v>23649844</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>269</v>
+        <v>193</v>
       </c>
       <c r="E10"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>271</v>
+        <v>195</v>
       </c>
       <c r="C11" s="2">
         <v>30192380</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>270</v>
+        <v>194</v>
       </c>
       <c r="E11"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C12" s="2">
         <v>23649844</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>207</v>
+        <v>132</v>
       </c>
       <c r="E12"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C13" s="8">
         <v>23649844</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>209</v>
+        <v>134</v>
       </c>
       <c r="E13"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C14" s="8">
         <v>23649844</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>272</v>
+        <v>196</v>
       </c>
       <c r="E14"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>277</v>
+        <v>201</v>
       </c>
       <c r="C15" s="8">
         <v>19151023</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>273</v>
+        <v>197</v>
       </c>
       <c r="E15"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>278</v>
+        <v>202</v>
       </c>
       <c r="C16" s="8">
         <v>24128683</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>275</v>
+        <v>199</v>
       </c>
       <c r="E16"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>279</v>
+        <v>203</v>
       </c>
       <c r="C17" s="8">
         <v>8042923</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>274</v>
+        <v>198</v>
       </c>
       <c r="E17"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>280</v>
+        <v>204</v>
       </c>
       <c r="C18" s="8">
         <v>6472420</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>276</v>
+        <v>200</v>
       </c>
       <c r="E18"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C19" s="2">
         <v>23649844</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>212</v>
+        <v>137</v>
       </c>
       <c r="E19"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C20" s="8">
         <v>23649844</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>213</v>
+        <v>138</v>
       </c>
       <c r="E20"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C21" s="10">
         <v>23649844</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>214</v>
+        <v>139</v>
       </c>
       <c r="E21"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C22" s="10">
         <v>23649844</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>216</v>
+        <v>141</v>
       </c>
       <c r="E22"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="6"/>
@@ -3526,7 +3301,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="6"/>
@@ -3534,7 +3309,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="6"/>
@@ -3542,7 +3317,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>66</v>
+        <v>42</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="6"/>
@@ -3550,7 +3325,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>185</v>
+        <v>112</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="6"/>
@@ -3558,22 +3333,22 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="C28" s="2">
         <v>30842973</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>281</v>
+        <v>205</v>
       </c>
       <c r="E28"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>186</v>
+        <v>113</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="6"/>
@@ -3581,22 +3356,22 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>187</v>
+        <v>114</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>251</v>
+        <v>176</v>
       </c>
       <c r="C30" s="2">
         <v>39910058</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>282</v>
+        <v>206</v>
       </c>
       <c r="E30"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>188</v>
+        <v>115</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="6"/>
@@ -3604,187 +3379,187 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>252</v>
+        <v>177</v>
       </c>
       <c r="C32" s="8">
         <v>19961535</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>283</v>
+        <v>207</v>
       </c>
       <c r="E32"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>288</v>
+        <v>212</v>
       </c>
       <c r="C33" s="8">
         <v>9225322</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>284</v>
+        <v>208</v>
       </c>
       <c r="E33"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>289</v>
+        <v>213</v>
       </c>
       <c r="C34" s="8">
         <v>25701871</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>285</v>
+        <v>209</v>
       </c>
       <c r="E34"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="C35" s="8">
         <v>24128683</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>286</v>
+        <v>210</v>
       </c>
       <c r="E35"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>268</v>
+        <v>192</v>
       </c>
       <c r="C36" s="8">
         <v>30842973</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>287</v>
+        <v>211</v>
       </c>
       <c r="E36"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>81</v>
+        <v>49</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C37" s="2">
         <v>23649844</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>291</v>
+        <v>215</v>
       </c>
       <c r="E37"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>81</v>
+        <v>49</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>251</v>
+        <v>176</v>
       </c>
       <c r="C38" s="2">
         <v>39910058</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>292</v>
+        <v>216</v>
       </c>
       <c r="E38"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>189</v>
+        <v>116</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>251</v>
+        <v>176</v>
       </c>
       <c r="C39" s="2">
         <v>39910058</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>290</v>
+        <v>214</v>
       </c>
       <c r="E39"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>92</v>
+        <v>55</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="C40" s="8">
         <v>30842973</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>293</v>
+        <v>217</v>
       </c>
       <c r="E40"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>92</v>
+        <v>55</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>257</v>
+        <v>182</v>
       </c>
       <c r="C41" s="8">
         <v>30697589</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>294</v>
+        <v>218</v>
       </c>
       <c r="E41"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>190</v>
+        <v>117</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>87</v>
+        <v>53</v>
       </c>
       <c r="C42" s="2">
         <v>40343075</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>227</v>
+        <v>152</v>
       </c>
       <c r="E42"/>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>113</v>
+        <v>68</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>253</v>
+        <v>178</v>
       </c>
       <c r="C43" s="8">
         <v>16951681</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>230</v>
+        <v>155</v>
       </c>
       <c r="E43"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>57</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" s="6"/>
@@ -3792,127 +3567,127 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>96</v>
+        <v>59</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C45" s="8">
         <v>23649844</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>295</v>
+        <v>219</v>
       </c>
       <c r="E45"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>59</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>297</v>
+        <v>221</v>
       </c>
       <c r="C46" s="8">
         <v>26896090</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>296</v>
+        <v>220</v>
       </c>
       <c r="E46"/>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>98</v>
+        <v>61</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C47" s="10">
         <v>23649844</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>233</v>
+        <v>158</v>
       </c>
       <c r="E47"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>254</v>
+        <v>179</v>
       </c>
       <c r="C48" s="8">
         <v>21909802</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>298</v>
+        <v>222</v>
       </c>
       <c r="E48"/>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>100</v>
+        <v>63</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C49" s="8">
         <v>23649844</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>299</v>
+        <v>223</v>
       </c>
       <c r="E49"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>102</v>
+        <v>65</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C50" s="10">
         <v>23649844</v>
       </c>
       <c r="D50" s="11" t="s">
-        <v>236</v>
+        <v>161</v>
       </c>
       <c r="E50"/>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>114</v>
+        <v>69</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C51" s="10">
         <v>23649844</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>237</v>
+        <v>162</v>
       </c>
       <c r="E51"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>115</v>
+        <v>70</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>255</v>
+        <v>180</v>
       </c>
       <c r="C52" s="8">
         <v>23261988</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>300</v>
+        <v>224</v>
       </c>
       <c r="E52"/>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>117</v>
+        <v>72</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" s="6"/>
@@ -3920,7 +3695,7 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>135</v>
+        <v>80</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" s="6"/>
@@ -3928,37 +3703,37 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>118</v>
+        <v>73</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>255</v>
+        <v>180</v>
       </c>
       <c r="C55" s="2">
         <v>23261988</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>240</v>
+        <v>165</v>
       </c>
       <c r="E55"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>119</v>
+        <v>74</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>256</v>
+        <v>181</v>
       </c>
       <c r="C56" s="8">
         <v>31695592</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>301</v>
+        <v>225</v>
       </c>
       <c r="E56"/>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>136</v>
+        <v>81</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" s="6"/>
@@ -3966,46 +3741,46 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>157</v>
+        <v>97</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>257</v>
+        <v>182</v>
       </c>
       <c r="C58" s="8">
         <v>30697589</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>244</v>
+        <v>169</v>
       </c>
       <c r="E58"/>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>158</v>
+        <v>98</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>257</v>
+        <v>182</v>
       </c>
       <c r="C59" s="8">
         <v>30697589</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>246</v>
+        <v>171</v>
       </c>
       <c r="E59"/>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>111</v>
+      </c>
+      <c r="B60" s="5" t="s">
         <v>182</v>
-      </c>
-      <c r="B60" s="5" t="s">
-        <v>257</v>
       </c>
       <c r="C60" s="8">
         <v>30697589</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>248</v>
+        <v>173</v>
       </c>
       <c r="E60"/>
     </row>
@@ -4085,563 +3860,6 @@
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A82" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B82" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="C82" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E82" s="5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A83" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B83" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="C83" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="D83" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A84" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B84" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="C84" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="D84" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A85" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B85" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C85" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D85" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E85" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A86" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B86" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C86" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="D86" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E86" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A87" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B87" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C87" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="D87" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A88" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B88" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C88" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="D88" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A89" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B89" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C89" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="D89" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="E89" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A90" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B90" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C90" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="D90" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A91" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B91" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="C91" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D91" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="E91" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A92" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B92" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="C92" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D92" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E92" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A93" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B93" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C93" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="D93" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A94" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A95" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A96" s="2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A97" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A98" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="B98" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="C98" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="D98" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="E98" s="5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A99" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="B99" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="C99" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="D99" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A100" s="2" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A101" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="B101" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="C101" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="D101" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="E101" s="5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A102" s="2" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A103" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B103" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="C103" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="D103" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="E103" s="5" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A104" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B104" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="C104" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="D104" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A105" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B105" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C105" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="D105" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A106" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="B106" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="C106" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="D106" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="E106" s="5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A107" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="B107" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="C107" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="D107" s="2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A108" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="B108" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C108" s="5" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A109" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B109" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="C109" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="D109" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="E109" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A110" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A111" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B111" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="C111" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="D111" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="E111" s="5" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A112" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B112" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C112" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="D112" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A113" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B113" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="C113" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="D113" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="E113" s="5" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A114" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="B114" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="C114" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="D114" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="E114" s="5" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A115" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="B115" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C115" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="D115" s="2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A116" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="C116" s="5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A117" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="B117" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C117" s="5" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A118" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A119" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="B119" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="C119" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="D119" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A120" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="B120" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="C120" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="D120" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="E120" s="5" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A121" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="D121" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A122" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="B122" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="C122" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="D122" s="2" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A123" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="B123" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="C123" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="D123" s="2" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A124" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="B124" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="C124" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="D124" s="2" t="s">
-        <v>183</v>
-      </c>
-    </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Inserted comment on whether pedigree is available
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\Krizchelle\ADLD Patient Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{446CB353-0879-4FB6-92C7-1AA6D3759734}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8854FAA-04C0-4DD7-BA95-C2C208B22596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -173,9 +173,6 @@
     <t>ADLD_del_1</t>
   </si>
   <si>
-    <t>Nmezi 2019</t>
-  </si>
-  <si>
     <t>Britain, England</t>
   </si>
   <si>
@@ -570,27 +567,9 @@
     <t>[Pyramidal signs] [Cerebellar signs] [Cognitive impairment]</t>
   </si>
   <si>
-    <t>Marklund 2008</t>
-  </si>
-  <si>
-    <t>Nmezi 2025</t>
-  </si>
-  <si>
-    <t>Giorgio 2015</t>
-  </si>
-  <si>
-    <t>Padiath 2006</t>
-  </si>
-  <si>
-    <t>DosSantos 2012</t>
-  </si>
-  <si>
     <t>Columbaro 2013</t>
   </si>
   <si>
-    <t>Zhang 2019</t>
-  </si>
-  <si>
     <t>Mezaki 2018</t>
   </si>
   <si>
@@ -618,9 +597,6 @@
     <t>Finnsson 2015</t>
   </si>
   <si>
-    <t>Sundblom 2009; Marklund 2006</t>
-  </si>
-  <si>
     <t>Alturkustani 2013</t>
   </si>
   <si>
@@ -648,18 +624,6 @@
     <t>Schwankhaus1988_1/56/F_Son; _1/56/F; _2/50/F; _3/60/F; _4/53/M; _5/56/M</t>
   </si>
   <si>
-    <t>Coffeen 2000</t>
-  </si>
-  <si>
-    <t>Padiath 2006; Alturkustani 2013</t>
-  </si>
-  <si>
-    <t>Alturkustani 2013_Eldridge</t>
-  </si>
-  <si>
-    <t>Schwankhaus 1988</t>
-  </si>
-  <si>
     <t>Nmezi2019_DEL3-1; Nmezi2019_DEL3-2; Nmezi2019_DEL3-3</t>
   </si>
   <si>
@@ -684,9 +648,6 @@
     <t>Bergui 1997</t>
   </si>
   <si>
-    <t>Brussino 2010</t>
-  </si>
-  <si>
     <t>Nmezi2025_F3-1; Nmezi2025_F3-2</t>
   </si>
   <si>
@@ -708,9 +669,6 @@
     <t>Terlizzi2016_IV11; Terlizzi2016_IV10; Terlizzi2016_IV12</t>
   </si>
   <si>
-    <t>Terlizzi 2016</t>
-  </si>
-  <si>
     <t>DosSantos2012_Proband; _Sister</t>
   </si>
   <si>
@@ -723,7 +681,49 @@
     <t>Zhang2019_II4_Proband; Zhang2019_II5</t>
   </si>
   <si>
-    <t>Meijer 2008</t>
+    <t>Coffeen 2000 *pedigree available</t>
+  </si>
+  <si>
+    <t>Brussino 2010 *pedigree available</t>
+  </si>
+  <si>
+    <t>DosSantos 2012 *pedigree available</t>
+  </si>
+  <si>
+    <t>Giorgio 2015 *pedigree available</t>
+  </si>
+  <si>
+    <t>Marklund 2008 *pedigree available</t>
+  </si>
+  <si>
+    <t>Meijer 2008 *pedigree available</t>
+  </si>
+  <si>
+    <t>Nmezi 2019 *pedigree available</t>
+  </si>
+  <si>
+    <t>Nmezi 2025 *pedigree available</t>
+  </si>
+  <si>
+    <t>Padiath 2006 *pedigree avialable; Alturkustani 2013</t>
+  </si>
+  <si>
+    <t>Padiath 2006 *pedigree available</t>
+  </si>
+  <si>
+    <t>Sundblom 2009 *pedigree available; Marklund 2006 *pedigree available</t>
+  </si>
+  <si>
+    <t>Terlizzi 2016 *pedigree available</t>
+  </si>
+  <si>
+    <t>Zhang 2019 *pedigree available</t>
+  </si>
+  <si>
+    <t>Alturkustani 2013; Eldridge 1984 *pedigree available</t>
+  </si>
+  <si>
+    <t>Schwankhaus 1988 *pedigree available</t>
   </si>
 </sst>
 </file>
@@ -1215,7 +1215,7 @@
         <v>10</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1238,7 +1238,7 @@
         <v>10</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1261,7 +1261,7 @@
         <v>10</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1307,7 +1307,7 @@
         <v>20</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1330,7 +1330,7 @@
         <v>10</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1376,7 +1376,7 @@
         <v>10</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1416,7 +1416,7 @@
         <v>10</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1461,7 +1461,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B16" s="2">
         <v>5</v>
@@ -1479,7 +1479,7 @@
         <v>10</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1499,15 +1499,15 @@
         <v>672515</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B18" s="2">
         <v>5</v>
@@ -1522,12 +1522,12 @@
         <v>4365976</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B19" s="2">
         <v>5</v>
@@ -1542,12 +1542,12 @@
         <v>4366000</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B20" s="2">
         <v>5</v>
@@ -1564,7 +1564,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B21" s="2">
         <v>5</v>
@@ -1581,7 +1581,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B22" s="2">
         <v>5</v>
@@ -1596,15 +1596,15 @@
         <v>608833</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B23" s="2">
         <v>5</v>
@@ -1619,15 +1619,15 @@
         <v>474998</v>
       </c>
       <c r="F23" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G23" s="5" t="s">
         <v>49</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B24" s="2">
         <v>5</v>
@@ -1644,7 +1644,7 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B25" s="2">
         <v>5</v>
@@ -1659,15 +1659,15 @@
         <v>250000</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B26" s="2">
         <v>5</v>
@@ -1682,12 +1682,12 @@
         <v>275347</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B27" s="2">
         <v>5</v>
@@ -1705,12 +1705,12 @@
         <v>10</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B28" s="2">
         <v>5</v>
@@ -1728,12 +1728,12 @@
         <v>10</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B29" s="2">
         <v>5</v>
@@ -1751,12 +1751,12 @@
         <v>10</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B30" s="2">
         <v>5</v>
@@ -1774,12 +1774,12 @@
         <v>10</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B31" s="2">
         <v>5</v>
@@ -1797,12 +1797,12 @@
         <v>10</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B32" s="2">
         <v>5</v>
@@ -1820,12 +1820,12 @@
         <v>10</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B33" s="2">
         <v>5</v>
@@ -1843,12 +1843,12 @@
         <v>10</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B34" s="2">
         <v>5</v>
@@ -1865,7 +1865,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B35" s="2">
         <v>5</v>
@@ -1882,7 +1882,7 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B36" s="2">
         <v>5</v>
@@ -1897,12 +1897,12 @@
         <v>156734</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B37" s="2">
         <v>5</v>
@@ -1919,7 +1919,7 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B38" s="2">
         <v>5</v>
@@ -1934,12 +1934,12 @@
         <v>59651</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B39" s="2">
         <v>5</v>
@@ -1957,12 +1957,12 @@
         <v>10</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B40" s="2">
         <v>5</v>
@@ -1974,12 +1974,12 @@
         <v>126903760</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B41" s="2">
         <v>5</v>
@@ -1991,12 +1991,12 @@
         <v>126896451</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B42" s="2">
         <v>5</v>
@@ -2030,7 +2030,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2038,7 +2038,7 @@
         <v>9</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2046,7 +2046,7 @@
         <v>13</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2054,7 +2054,7 @@
         <v>16</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2062,7 +2062,7 @@
         <v>17</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2070,7 +2070,7 @@
         <v>18</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2078,7 +2078,7 @@
         <v>19</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2086,7 +2086,7 @@
         <v>28</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2094,7 +2094,7 @@
         <v>29</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2102,7 +2102,7 @@
         <v>30</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2110,7 +2110,7 @@
         <v>31</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2118,7 +2118,7 @@
         <v>37</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2126,7 +2126,7 @@
         <v>38</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2134,7 +2134,7 @@
         <v>39</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2142,15 +2142,15 @@
         <v>41</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2158,207 +2158,207 @@
         <v>43</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -2385,7 +2385,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>7</v>
@@ -2394,10 +2394,10 @@
         <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>120</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2411,10 +2411,10 @@
         <v>16</v>
       </c>
       <c r="E2" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="F2" t="s">
         <v>125</v>
-      </c>
-      <c r="F2" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -2431,10 +2431,10 @@
         <v>45</v>
       </c>
       <c r="E3" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="F3" t="s">
         <v>127</v>
-      </c>
-      <c r="F3" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -2451,10 +2451,10 @@
         <v>43</v>
       </c>
       <c r="E4" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="F4" t="s">
         <v>129</v>
-      </c>
-      <c r="F4" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -2468,7 +2468,7 @@
         <v>3</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -2479,7 +2479,7 @@
         <v>23</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -2496,10 +2496,10 @@
         <v>26</v>
       </c>
       <c r="E7" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="F7" t="s">
         <v>134</v>
-      </c>
-      <c r="F7" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -2510,7 +2510,7 @@
         <v>23</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -2527,7 +2527,7 @@
         <v>33</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -2544,10 +2544,10 @@
         <v>35</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -2558,10 +2558,10 @@
         <v>23</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -2586,7 +2586,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>42</v>
@@ -2597,24 +2597,24 @@
         <v>43</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C17" s="2">
         <v>3</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E17" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="F17" t="s">
         <v>141</v>
-      </c>
-      <c r="F17" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>23</v>
@@ -2622,46 +2622,46 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C19" s="2">
         <v>5</v>
       </c>
       <c r="E19" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="F19" t="s">
         <v>143</v>
-      </c>
-      <c r="F19" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C21" s="2">
         <v>32</v>
       </c>
       <c r="E21" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="F21" t="s">
         <v>145</v>
-      </c>
-      <c r="F21" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C22" s="2">
         <v>1</v>
@@ -2670,43 +2670,43 @@
         <v>52</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F22" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F24" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C25" s="2">
         <v>1</v>
@@ -2715,70 +2715,70 @@
         <v>34</v>
       </c>
       <c r="E25" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="F25" t="s">
         <v>149</v>
-      </c>
-      <c r="F25" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E26" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="F26" t="s">
         <v>152</v>
-      </c>
-      <c r="F26" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="D29" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>106</v>
-      </c>
       <c r="E29" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="F29" t="s">
         <v>155</v>
-      </c>
-      <c r="F29" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>34</v>
@@ -2790,75 +2790,75 @@
         <v>45</v>
       </c>
       <c r="E31" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="F31" t="s">
         <v>158</v>
-      </c>
-      <c r="F31" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C32" s="2">
         <v>8</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E34" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="F34" t="s">
         <v>162</v>
-      </c>
-      <c r="F34" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F37" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C38" s="2">
         <v>2</v>
@@ -2867,26 +2867,26 @@
         <v>58</v>
       </c>
       <c r="E38" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="F38" t="s">
         <v>166</v>
-      </c>
-      <c r="F38" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C40" s="2">
         <v>6</v>
@@ -2895,50 +2895,50 @@
         <v>44</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F40" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>98</v>
       </c>
       <c r="C41" s="2">
         <v>6</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F41" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C42" s="2">
         <v>6</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F42" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -2952,9 +2952,9 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="32.5703125" style="5" customWidth="1"/>
-    <col min="3" max="3" width="57.28515625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="255.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="52.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="139.85546875" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2962,13 +2962,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>123</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -2982,7 +2982,7 @@
         <v>23649844</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -2990,13 +2990,13 @@
         <v>9</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C3" s="2">
         <v>19001169</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -3004,13 +3004,13 @@
         <v>13</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>174</v>
+        <v>215</v>
       </c>
       <c r="C4" s="2">
         <v>16823806</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -3018,13 +3018,13 @@
         <v>13</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="C5" s="2">
         <v>26053668</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -3038,7 +3038,7 @@
         <v>23649844</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -3046,13 +3046,13 @@
         <v>13</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>190</v>
+        <v>221</v>
       </c>
       <c r="C7" s="2">
         <v>18945794</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -3060,13 +3060,13 @@
         <v>13</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="C8" s="2">
         <v>24128683</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -3074,7 +3074,7 @@
         <v>16</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="C9" s="2">
         <v>26053668</v>
@@ -3092,7 +3092,7 @@
         <v>23649844</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -3100,13 +3100,13 @@
         <v>16</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="C11" s="2">
         <v>30192380</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -3120,7 +3120,7 @@
         <v>23649844</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -3134,7 +3134,7 @@
         <v>23649844</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -3148,7 +3148,7 @@
         <v>23649844</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -3156,13 +3156,13 @@
         <v>19</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="C15" s="8">
         <v>19151023</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -3170,13 +3170,13 @@
         <v>19</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>201</v>
+        <v>219</v>
       </c>
       <c r="C16" s="8">
         <v>24128683</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -3184,13 +3184,13 @@
         <v>19</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>202</v>
+        <v>224</v>
       </c>
       <c r="C17" s="8">
         <v>8042923</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -3198,13 +3198,13 @@
         <v>19</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>203</v>
+        <v>225</v>
       </c>
       <c r="C18" s="8">
         <v>6472420</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -3218,7 +3218,7 @@
         <v>23649844</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -3232,7 +3232,7 @@
         <v>23649844</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -3246,7 +3246,7 @@
         <v>23649844</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -3260,7 +3260,7 @@
         <v>23649844</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -3293,7 +3293,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="6"/>
@@ -3303,74 +3303,74 @@
         <v>43</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>44</v>
+        <v>217</v>
       </c>
       <c r="C28" s="2">
         <v>30842973</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="6"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>175</v>
+        <v>218</v>
       </c>
       <c r="C30" s="2">
         <v>39910058</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="6"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>176</v>
+        <v>214</v>
       </c>
       <c r="C32" s="8">
         <v>19961535</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="C33" s="8">
         <v>9225322</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B34" s="9" t="s">
         <v>212</v>
@@ -3379,40 +3379,40 @@
         <v>25701871</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>44</v>
+        <v>217</v>
       </c>
       <c r="C35" s="8">
         <v>24128683</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="C36" s="8">
         <v>30842973</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>27</v>
@@ -3421,103 +3421,103 @@
         <v>23649844</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>214</v>
+        <v>201</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>175</v>
+        <v>218</v>
       </c>
       <c r="C38" s="2">
         <v>39910058</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>215</v>
+        <v>202</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>175</v>
+        <v>218</v>
       </c>
       <c r="C39" s="2">
         <v>39910058</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>213</v>
+        <v>200</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>54</v>
-      </c>
-      <c r="B40" s="5" t="s">
-        <v>44</v>
+        <v>53</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>217</v>
       </c>
       <c r="C40" s="8">
         <v>30842973</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>216</v>
+        <v>203</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="C41" s="8">
         <v>30697589</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>217</v>
+        <v>204</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C42" s="2">
         <v>40343075</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>177</v>
+        <v>220</v>
       </c>
       <c r="C43" s="8">
         <v>16951681</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" s="6"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>27</v>
@@ -3526,26 +3526,26 @@
         <v>23649844</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>218</v>
+        <v>205</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C46" s="8">
         <v>26896090</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B47" s="5" t="s">
         <v>27</v>
@@ -3554,26 +3554,26 @@
         <v>23649844</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>178</v>
+        <v>213</v>
       </c>
       <c r="C48" s="8">
         <v>21909802</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B49" s="5" t="s">
         <v>27</v>
@@ -3582,12 +3582,12 @@
         <v>23649844</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>222</v>
+        <v>208</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B50" s="5" t="s">
         <v>27</v>
@@ -3596,12 +3596,12 @@
         <v>23649844</v>
       </c>
       <c r="D50" s="11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>27</v>
@@ -3610,112 +3610,112 @@
         <v>23649844</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="C52" s="8">
         <v>23261988</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>223</v>
+        <v>209</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" s="6"/>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" s="6"/>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="C55" s="2">
         <v>23261988</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="C56" s="8">
         <v>31695592</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>224</v>
+        <v>210</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" s="6"/>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="C58" s="8">
         <v>30697589</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="C59" s="8">
         <v>30697589</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="C60" s="8">
         <v>30697589</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated case reported names in Excel sheet
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\Krizchelle\ADLD Patient Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8854FAA-04C0-4DD7-BA95-C2C208B22596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90DFE790-6F95-4BAD-973B-3F7D4C7056BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="223">
   <si>
     <t>Item name</t>
   </si>
@@ -437,34 +437,16 @@
 [MRI abnormality, Grade 5]</t>
   </si>
   <si>
-    <t>Giorgio2013_A4</t>
-  </si>
-  <si>
     <t>[Symptomatic - specific symptoms not documented]</t>
   </si>
   <si>
-    <t>Giorgio2013_A5</t>
-  </si>
-  <si>
     <t>[Autonomic dysfunction] [Orthostatic hypotension] [Bladder/bowel dysfunction] [Thermoregulatory dysfunction] [Pyramidal signs] [Cerebellar signs] [Sexual dysfunction]</t>
   </si>
   <si>
     <t>[Cerebral white matter abnormalities (MRI), symmetric] [Cerebellar white matter lesions (MRI), symmetric] [Cerebellar white matter lesions (MRI)]  [Spinal cord abnormalities (MRI)] [Cerebellar white matter lesions (CT), symmetric] [Cerebral white matter abnormalities (CT)] [Cerebellar white matter lesions (CT)] [Spinal cord abnormalities (CT)]</t>
   </si>
   <si>
-    <t>Giorgio2013_A8,AV1</t>
-  </si>
-  <si>
-    <t>Giorgio2013_A10</t>
-  </si>
-  <si>
-    <t>Giorgio2013_A11</t>
-  </si>
-  <si>
     <t>Not reported / unknown.</t>
-  </si>
-  <si>
-    <t>Giorgio2013_A14</t>
   </si>
   <si>
     <t xml:space="preserve">[Pyramidal signs] [Cerebellar signs] [Dysarthria] [Autonomic dysfunction] [Bladder/bowel dysfunction] [Pseudobulbar affect]
@@ -498,48 +480,30 @@
     <t>[Cerebral white matter abnormalities (MRI)] [Cerebellar white matter lesions (MRI)]</t>
   </si>
   <si>
-    <t>Wang2025_Proband</t>
-  </si>
-  <si>
     <t>[Autonomic dysfunction] [Bladder/bowel dysfunction] [Pyramidal signs] [Dysphagia]</t>
   </si>
   <si>
     <t>[Cerebral white matter abnormalities (MRI), possibly symmetric] [Cerebellar white matter lesions (MRI), possibly symmetric]</t>
   </si>
   <si>
-    <t>Padiath2006_K50069</t>
-  </si>
-  <si>
     <t>[Autonomic dysfunction] [Orthostatic hypotension] [Bladder/bowel dysfunction] [Sexual dysfunction] [Pyramidal signs] [Cerebellar signs] [Dysphagia] [Possible Pseudobulbar affect]</t>
   </si>
   <si>
     <t>[Cerebellar white matter lesions (MRI)]</t>
   </si>
   <si>
-    <t>Giorgio2013_FR1,FR2</t>
-  </si>
-  <si>
     <t>[Autonomic dysfunction] [Bladder/bowel dysfunction] [Pyramidal signs] [Cerebellar signs] [Pseudobulbar affect] [Cognitive impairment]</t>
   </si>
   <si>
     <t>[Cerebral white matter abnormalities (MRI), symmetric] [Cerebellar white matter lesions (MRI)] [Spinal cord abnormalities (MRI)]</t>
   </si>
   <si>
-    <t>Giorgio2013_IT1</t>
-  </si>
-  <si>
-    <t>Giorgio2013_IT2</t>
-  </si>
-  <si>
     <t>[Autonomic dysfunction] [Orthostatic hypotension] [Bladder/bowel dysfunction] [Sexual dysfunction] [Thermoregulatory dysfunction] [Pyramidal signs] [Cerebellar signs]</t>
   </si>
   <si>
     <t>[Cerebral white matter abnormalities (MRI)]</t>
   </si>
   <si>
-    <t>Columbaro2013_ADLD2</t>
-  </si>
-  <si>
     <t>[Autonomic dysfunction] [Orthostatic hypotension] [Sexual dysfunction]</t>
   </si>
   <si>
@@ -549,21 +513,12 @@
     <t>[Cerebral white matter abnormalities (MRI), symmetric] [Cerebellar white matter lesions (MRI), symmetric] [Spinal cord abnormalities (MRI)]</t>
   </si>
   <si>
-    <t>Mezaki2018_PedigreeI_Patient1</t>
-  </si>
-  <si>
     <t>[Autonomic dysfunction] [Orthostatic hypotension] [Bladder/bowel dysfunction] [Thermoregulatory dysfunction] [Pyramidal signs] [Cerebellar signs] [Cognitive impairment]</t>
   </si>
   <si>
-    <t>Mezaki2018_PedigreeII_Patient2</t>
-  </si>
-  <si>
     <t>[Autonomic dysfunction] [Orthostatic hypotension] [Bladder/bowel dysfunction] [Pyramidal signs] [Cerebellar signs] [Cognitive impairment]</t>
   </si>
   <si>
-    <t>Mezaki2018_PedigreeIII_Patient4</t>
-  </si>
-  <si>
     <t>[Pyramidal signs] [Cerebellar signs] [Cognitive impairment]</t>
   </si>
   <si>
@@ -573,114 +528,18 @@
     <t>Mezaki 2018</t>
   </si>
   <si>
-    <t>Giorgio2013_A1</t>
-  </si>
-  <si>
-    <t>Meijer2008_IV1; _II3; _II4; _III10; _IV13; _IV4</t>
-  </si>
-  <si>
-    <t>Marklund2008_Cohort</t>
-  </si>
-  <si>
-    <t>Finnsson2015_Family1_23F; _22M; _20M; _19F; _18F; _17F; _16F; _15M; _14F; _13F; _12F; _11M; _10M; _8F; _7F; _5M; _4M; _3M; _2M; _1F</t>
-  </si>
-  <si>
-    <t>Giorgio2013_A2</t>
-  </si>
-  <si>
-    <t>Sundblom2009_1; Marklund2006</t>
-  </si>
-  <si>
-    <t>Alturkustani2013_Sundlom_7</t>
-  </si>
-  <si>
     <t>Finnsson 2015</t>
   </si>
   <si>
     <t>Alturkustani 2013</t>
   </si>
   <si>
-    <t>Giorgio2013_A3</t>
-  </si>
-  <si>
-    <t>Finnsson2019_Family2_5; _6</t>
-  </si>
-  <si>
     <t>Finnsson 2019</t>
   </si>
   <si>
-    <t>Giorgio2013_A6,A7,K2-3</t>
-  </si>
-  <si>
-    <t>Coffeen2000_K2685</t>
-  </si>
-  <si>
-    <t>Alturkustani2013_Eldridge_1</t>
-  </si>
-  <si>
-    <t>Padiath2006_K4233; Alturkustani2013_Coffeen_3</t>
-  </si>
-  <si>
-    <t>Schwankhaus1988_1/56/F_Son; _1/56/F; _2/50/F; _3/60/F; _4/53/M; _5/56/M</t>
-  </si>
-  <si>
-    <t>Nmezi2019_DEL3-1; Nmezi2019_DEL3-2; Nmezi2019_DEL3-3</t>
-  </si>
-  <si>
-    <t>Nmezi2025_F1-1; Nmezi2025_F1-2; Nmezi2025_F1-3; Nmezi2025_F1-4; Nmezi2025_F1-5</t>
-  </si>
-  <si>
-    <t>Giorgio2015_ADLD-1-TO</t>
-  </si>
-  <si>
-    <t>Bergui1997_Family1</t>
-  </si>
-  <si>
-    <t>Brussino2010_ADLD-1-TO</t>
-  </si>
-  <si>
-    <t>Nmezi2019_DEL2-1</t>
-  </si>
-  <si>
-    <t>Alturkustani2013</t>
-  </si>
-  <si>
     <t>Bergui 1997</t>
   </si>
   <si>
-    <t>Nmezi2025_F3-1; Nmezi2025_F3-2</t>
-  </si>
-  <si>
-    <t>Giorgio2013_BR1</t>
-  </si>
-  <si>
-    <t>Nmezi2025_F4-1</t>
-  </si>
-  <si>
-    <t>Nmezi2019_DEL1-1</t>
-  </si>
-  <si>
-    <t>Mezaki2018_PedigreeIV_Patient5; Mezaki2018_PedigreeIV_Patient6</t>
-  </si>
-  <si>
-    <t>Giorgio2013_IT3</t>
-  </si>
-  <si>
-    <t>Terlizzi2016_IV11; Terlizzi2016_IV10; Terlizzi2016_IV12</t>
-  </si>
-  <si>
-    <t>DosSantos2012_Proband; _Sister</t>
-  </si>
-  <si>
-    <t>Giorgio2013_G1</t>
-  </si>
-  <si>
-    <t>Columbaro2013_ADLD1; Columbaro2013_ADLD3</t>
-  </si>
-  <si>
-    <t>Zhang2019_II4_Proband; Zhang2019_II5</t>
-  </si>
-  <si>
     <t>Coffeen 2000 *pedigree available</t>
   </si>
   <si>
@@ -724,6 +583,138 @@
   </si>
   <si>
     <t>Schwankhaus 1988 *pedigree available</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>A3</t>
+  </si>
+  <si>
+    <t>A11</t>
+  </si>
+  <si>
+    <t>A14</t>
+  </si>
+  <si>
+    <t>Cohort</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>Patient 1</t>
+  </si>
+  <si>
+    <t>Patient 7</t>
+  </si>
+  <si>
+    <t>A4</t>
+  </si>
+  <si>
+    <t>A5</t>
+  </si>
+  <si>
+    <t>A6, A7, K2-3</t>
+  </si>
+  <si>
+    <t>Family2_5, _6</t>
+  </si>
+  <si>
+    <t>Family1_23F, _22M, _20M, _19F, _18F, _17F, _16F, _15M, _14F, _13F, _12F, _11M, _10M, _8F, _7F, _5M, _4M, _3M, _2M, _1F</t>
+  </si>
+  <si>
+    <t>IV1, II3, II4, III10, IV13, IV4</t>
+  </si>
+  <si>
+    <t>K2685</t>
+  </si>
+  <si>
+    <t>K4233, Alturkustani2013_Coffeen_3</t>
+  </si>
+  <si>
+    <t>1/56/F_Son, _1/56/F, _2/50/F, _3/60/F, _4/53/M, _5/56/M</t>
+  </si>
+  <si>
+    <t>A8, AV1</t>
+  </si>
+  <si>
+    <t>A10</t>
+  </si>
+  <si>
+    <t>DEL3-1, DEL3-2, DEL3-3</t>
+  </si>
+  <si>
+    <t>F1-1, F1-2, F1-3, F1-4, F1-5</t>
+  </si>
+  <si>
+    <t>ADLD-1-TO</t>
+  </si>
+  <si>
+    <t>Family 1</t>
+  </si>
+  <si>
+    <t>DEL2-1</t>
+  </si>
+  <si>
+    <t>BR1</t>
+  </si>
+  <si>
+    <t>F4-1</t>
+  </si>
+  <si>
+    <t>F3-1, F3-2</t>
+  </si>
+  <si>
+    <t>DEL1-1</t>
+  </si>
+  <si>
+    <t>PedigreeIV_Patient5, PedigreeIV_Patient6</t>
+  </si>
+  <si>
+    <t>Proband</t>
+  </si>
+  <si>
+    <t>K50069</t>
+  </si>
+  <si>
+    <t>IT3</t>
+  </si>
+  <si>
+    <t>IV11, IV10, IV12</t>
+  </si>
+  <si>
+    <t>FR1, FR2</t>
+  </si>
+  <si>
+    <t>Proband, Sister</t>
+  </si>
+  <si>
+    <t>G1</t>
+  </si>
+  <si>
+    <t>IT1</t>
+  </si>
+  <si>
+    <t>IT2</t>
+  </si>
+  <si>
+    <t>ADLD1, ADLD3</t>
+  </si>
+  <si>
+    <t>ADLD2</t>
+  </si>
+  <si>
+    <t>II4_Proband, II5</t>
+  </si>
+  <si>
+    <t>PedigreeI_Patient1</t>
+  </si>
+  <si>
+    <t>PedigreeII_Patient2</t>
+  </si>
+  <si>
+    <t>PedigreeIII_Patient4</t>
   </si>
 </sst>
 </file>
@@ -2468,7 +2459,7 @@
         <v>3</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -2479,7 +2470,7 @@
         <v>23</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -2496,10 +2487,10 @@
         <v>26</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F7" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -2510,7 +2501,7 @@
         <v>23</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -2527,7 +2518,7 @@
         <v>33</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -2544,10 +2535,10 @@
         <v>35</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F10" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -2558,10 +2549,10 @@
         <v>23</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F11" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -2606,10 +2597,10 @@
         <v>99</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="F17" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -2631,10 +2622,10 @@
         <v>5</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="F19" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -2650,10 +2641,10 @@
         <v>32</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="F21" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -2670,10 +2661,10 @@
         <v>52</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="F22" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -2695,10 +2686,10 @@
         <v>102</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="F24" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -2715,10 +2706,10 @@
         <v>34</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="F25" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -2726,10 +2717,10 @@
         <v>115</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="F26" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -2737,7 +2728,7 @@
         <v>66</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -2759,10 +2750,10 @@
         <v>105</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="F29" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -2773,7 +2764,7 @@
         <v>65</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -2790,10 +2781,10 @@
         <v>45</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="F31" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -2810,7 +2801,7 @@
         <v>76</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -2818,7 +2809,7 @@
         <v>67</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -2826,10 +2817,10 @@
         <v>68</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="F34" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -2847,10 +2838,10 @@
         <v>71</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="F37" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -2867,10 +2858,10 @@
         <v>58</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="F38" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -2895,10 +2886,10 @@
         <v>44</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>168</v>
+        <v>155</v>
       </c>
       <c r="F40" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2915,10 +2906,10 @@
         <v>101</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>170</v>
+        <v>156</v>
       </c>
       <c r="F41" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -2935,10 +2926,10 @@
         <v>101</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="F42" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -2982,7 +2973,7 @@
         <v>23649844</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -2990,13 +2981,13 @@
         <v>9</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>216</v>
+        <v>169</v>
       </c>
       <c r="C3" s="2">
         <v>19001169</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -3004,13 +2995,13 @@
         <v>13</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>215</v>
+        <v>168</v>
       </c>
       <c r="C4" s="2">
         <v>16823806</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -3018,13 +3009,13 @@
         <v>13</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>182</v>
+        <v>160</v>
       </c>
       <c r="C5" s="2">
         <v>26053668</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -3038,7 +3029,7 @@
         <v>23649844</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -3046,13 +3037,13 @@
         <v>13</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>221</v>
+        <v>174</v>
       </c>
       <c r="C7" s="2">
         <v>18945794</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -3060,13 +3051,13 @@
         <v>13</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>183</v>
+        <v>161</v>
       </c>
       <c r="C8" s="2">
         <v>24128683</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -3074,7 +3065,7 @@
         <v>16</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>182</v>
+        <v>160</v>
       </c>
       <c r="C9" s="2">
         <v>26053668</v>
@@ -3092,7 +3083,7 @@
         <v>23649844</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -3100,13 +3091,13 @@
         <v>16</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>186</v>
+        <v>162</v>
       </c>
       <c r="C11" s="2">
         <v>30192380</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -3120,7 +3111,7 @@
         <v>23649844</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>130</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -3134,7 +3125,7 @@
         <v>23649844</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>132</v>
+        <v>188</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -3148,7 +3139,7 @@
         <v>23649844</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -3156,13 +3147,13 @@
         <v>19</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>211</v>
+        <v>164</v>
       </c>
       <c r="C15" s="8">
         <v>19151023</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -3170,13 +3161,13 @@
         <v>19</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>219</v>
+        <v>172</v>
       </c>
       <c r="C16" s="8">
         <v>24128683</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -3184,13 +3175,13 @@
         <v>19</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>224</v>
+        <v>177</v>
       </c>
       <c r="C17" s="8">
         <v>8042923</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -3198,13 +3189,13 @@
         <v>19</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>225</v>
+        <v>178</v>
       </c>
       <c r="C18" s="8">
         <v>6472420</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -3218,7 +3209,7 @@
         <v>23649844</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>135</v>
+        <v>196</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -3232,7 +3223,7 @@
         <v>23649844</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>136</v>
+        <v>197</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -3246,7 +3237,7 @@
         <v>23649844</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>137</v>
+        <v>181</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -3260,7 +3251,7 @@
         <v>23649844</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>139</v>
+        <v>182</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -3303,13 +3294,13 @@
         <v>43</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>217</v>
+        <v>170</v>
       </c>
       <c r="C28" s="2">
         <v>30842973</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -3324,13 +3315,13 @@
         <v>112</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>218</v>
+        <v>171</v>
       </c>
       <c r="C30" s="2">
         <v>39910058</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -3345,13 +3336,13 @@
         <v>45</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>214</v>
+        <v>167</v>
       </c>
       <c r="C32" s="8">
         <v>19961535</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -3359,13 +3350,13 @@
         <v>45</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>199</v>
+        <v>163</v>
       </c>
       <c r="C33" s="8">
         <v>9225322</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -3373,13 +3364,13 @@
         <v>45</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>212</v>
+        <v>165</v>
       </c>
       <c r="C34" s="8">
         <v>25701871</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -3387,13 +3378,13 @@
         <v>46</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>217</v>
+        <v>170</v>
       </c>
       <c r="C35" s="8">
         <v>24128683</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -3401,13 +3392,13 @@
         <v>46</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>183</v>
+        <v>161</v>
       </c>
       <c r="C36" s="8">
         <v>30842973</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>198</v>
+        <v>185</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -3421,7 +3412,7 @@
         <v>23649844</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -3429,13 +3420,13 @@
         <v>47</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>218</v>
+        <v>171</v>
       </c>
       <c r="C38" s="2">
         <v>39910058</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -3443,13 +3434,13 @@
         <v>114</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>218</v>
+        <v>171</v>
       </c>
       <c r="C39" s="2">
         <v>39910058</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -3457,13 +3448,13 @@
         <v>53</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>217</v>
+        <v>170</v>
       </c>
       <c r="C40" s="8">
         <v>30842973</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -3471,13 +3462,13 @@
         <v>53</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="C41" s="8">
         <v>30697589</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -3491,7 +3482,7 @@
         <v>40343075</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>150</v>
+        <v>208</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -3499,13 +3490,13 @@
         <v>66</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>220</v>
+        <v>173</v>
       </c>
       <c r="C43" s="8">
         <v>16951681</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>153</v>
+        <v>209</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -3526,7 +3517,7 @@
         <v>23649844</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -3534,13 +3525,13 @@
         <v>57</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>222</v>
+        <v>175</v>
       </c>
       <c r="C46" s="8">
         <v>26896090</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -3554,7 +3545,7 @@
         <v>23649844</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>156</v>
+        <v>212</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -3562,13 +3553,13 @@
         <v>61</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>213</v>
+        <v>166</v>
       </c>
       <c r="C48" s="8">
         <v>21909802</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -3582,7 +3573,7 @@
         <v>23649844</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -3596,7 +3587,7 @@
         <v>23649844</v>
       </c>
       <c r="D50" s="11" t="s">
-        <v>159</v>
+        <v>215</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -3610,7 +3601,7 @@
         <v>23649844</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>160</v>
+        <v>216</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -3618,13 +3609,13 @@
         <v>68</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="C52" s="8">
         <v>23261988</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -3646,13 +3637,13 @@
         <v>71</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="C55" s="2">
         <v>23261988</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>163</v>
+        <v>218</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -3660,13 +3651,13 @@
         <v>72</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>223</v>
+        <v>176</v>
       </c>
       <c r="C56" s="8">
         <v>31695592</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -3681,13 +3672,13 @@
         <v>95</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="C58" s="8">
         <v>30697589</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>167</v>
+        <v>220</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -3695,13 +3686,13 @@
         <v>96</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="C59" s="8">
         <v>30697589</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>169</v>
+        <v>221</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -3709,13 +3700,13 @@
         <v>109</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="C60" s="8">
         <v>30697589</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>171</v>
+        <v>222</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated evidence section of master list
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\Krizchelle\ADLD Patient Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90DFE790-6F95-4BAD-973B-3F7D4C7056BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2639C71F-E11E-4CEC-BBAE-B904DDA99923}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Molecular" sheetId="4" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="243">
   <si>
     <t>Item name</t>
   </si>
@@ -390,14 +390,6 @@
   </si>
   <si>
     <t>Summary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">publications
-literature case labels
-multigenerational family
-estimated unique individuals
-high-confidence linked individuals
-Deduplication status: </t>
   </si>
   <si>
     <t>Country of origin</t>
@@ -715,6 +707,135 @@
   </si>
   <si>
     <t>PedigreeIII_Patient4</t>
+  </si>
+  <si>
+    <t>2 publications
+7 literature case labels
+Multigenerational family - 4 generations
+16 estimated unique individuals
+Deduplication status: partially resolved</t>
+  </si>
+  <si>
+    <t>5 publications
+24 literature case labels
+Multigenerational family - 6 generations
+31 estimated unique individuals
+Deduplication status: partially resolved</t>
+  </si>
+  <si>
+    <t>8 publications
+24 literature case labels
+Multigenerational family - 6 generations
+31 estimated unique individuals
+Deduplication status: partially resolved</t>
+  </si>
+  <si>
+    <t>3 publications
+4 literature case labels
+4 estimated unique individuals
+Deduplication status: partially resolved</t>
+  </si>
+  <si>
+    <t>1 publication
+1 literature case labels
+1 estimated unique individuals
+Deduplication status: resolved</t>
+  </si>
+  <si>
+    <t>5 publications
+13 literature case labels
+Multigenerational family - 5 generations
+13 estimated unique individuals
+Deduplication status: partially resolved</t>
+  </si>
+  <si>
+    <t>1 publications
+2 literature case labels
+2 estimated unique individuals
+Deduplication status: resolved</t>
+  </si>
+  <si>
+    <t>1 publications
+1 literature case labels
+1 estimated unique individuals
+Deduplication status: resolved</t>
+  </si>
+  <si>
+    <t>? publications
+? literature case labels
+Multigenerational family?
+? estimated unique individuals
+Deduplication status: ?</t>
+  </si>
+  <si>
+    <t>1 publications
+3 literature case labels
+Deduplication status: partially resolved</t>
+  </si>
+  <si>
+    <t>1 publications
+3 literature case labels
+3 estimated unique individuals
+Deduplication status: resolved</t>
+  </si>
+  <si>
+    <t>1 publications
+5 literature case labels
+5 estimated unique individuals
+Deduplication status: resolved</t>
+  </si>
+  <si>
+    <t>3 publications
+3 literature case labels
+Multigenerational family - 7 generations
+2 estimated unique individuals
+Deduplication status: partially resolved</t>
+  </si>
+  <si>
+    <t>2 publications
+2 literature case labels
+1 estimated unique individuals
+Deduplication status: partially resolved</t>
+  </si>
+  <si>
+    <t>2 publications
+2 literature case labels
+Deduplication status: partially resolved</t>
+  </si>
+  <si>
+    <t>2 publications
+23 literature case labels
+Deduplication status: partially resolved</t>
+  </si>
+  <si>
+    <t>1 publications
+1 literature case labels
+Multigenerational family - 2 generations
+Deduplication status: resolved</t>
+  </si>
+  <si>
+    <t>2 publications
+4 literature case labels
+Multigenerational family - 5 generations
+3 estimated unique individuals
+Deduplication status: partially resolved</t>
+  </si>
+  <si>
+    <t>2 publications
+3 literature case labels
+Multigenerational family - 5 generations
+1 estimated unique individuals
+Deduplication status: partially resolved</t>
+  </si>
+  <si>
+    <t>1 publications
+1 literature case labels
+Deduplication status: resolved</t>
+  </si>
+  <si>
+    <t>1 publications
+2 literature case labels
+Deduplication status: resolved</t>
   </si>
 </sst>
 </file>
@@ -2009,6 +2130,9 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93210A17-976E-449D-A8F5-248F94CB6DA5}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:B42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2024,342 +2148,322 @@
         <v>116</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>28</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+      <c r="B12" s="7"/>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+      <c r="B13" s="7"/>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B14" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+      <c r="B14" s="7"/>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+      <c r="B15" s="7"/>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B16" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+      <c r="B16" s="7"/>
+    </row>
+    <row r="17" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>111</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B19" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+      <c r="B19" s="7"/>
+    </row>
+    <row r="20" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>113</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+      <c r="B21" s="7"/>
+    </row>
+    <row r="22" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>46</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>47</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>114</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>53</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>115</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>66</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B29" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+      <c r="B29" s="7"/>
+    </row>
+    <row r="30" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>59</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>61</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>67</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>68</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>70</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>78</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>72</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B39" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+      <c r="B39" s="7"/>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B40" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+      <c r="B40" s="7"/>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B41" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+      <c r="B41" s="7"/>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B42" s="7" t="s">
-        <v>117</v>
-      </c>
+      <c r="B42" s="7"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup scale="86" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2376,7 +2480,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>7</v>
@@ -2385,10 +2489,10 @@
         <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>119</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2402,10 +2506,10 @@
         <v>16</v>
       </c>
       <c r="E2" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="F2" t="s">
         <v>124</v>
-      </c>
-      <c r="F2" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -2422,10 +2526,10 @@
         <v>45</v>
       </c>
       <c r="E3" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="F3" t="s">
         <v>126</v>
-      </c>
-      <c r="F3" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -2442,10 +2546,10 @@
         <v>43</v>
       </c>
       <c r="E4" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="F4" t="s">
         <v>128</v>
-      </c>
-      <c r="F4" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -2459,7 +2563,7 @@
         <v>3</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -2470,7 +2574,7 @@
         <v>23</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -2487,10 +2591,10 @@
         <v>26</v>
       </c>
       <c r="E7" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="F7" t="s">
         <v>131</v>
-      </c>
-      <c r="F7" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -2501,7 +2605,7 @@
         <v>23</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -2518,7 +2622,7 @@
         <v>33</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -2535,10 +2639,10 @@
         <v>35</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -2549,10 +2653,10 @@
         <v>23</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -2597,10 +2701,10 @@
         <v>99</v>
       </c>
       <c r="E17" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="F17" t="s">
         <v>134</v>
-      </c>
-      <c r="F17" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -2622,10 +2726,10 @@
         <v>5</v>
       </c>
       <c r="E19" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F19" t="s">
         <v>136</v>
-      </c>
-      <c r="F19" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -2641,10 +2745,10 @@
         <v>32</v>
       </c>
       <c r="E21" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="F21" t="s">
         <v>138</v>
-      </c>
-      <c r="F21" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -2661,10 +2765,10 @@
         <v>52</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F22" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -2675,7 +2779,7 @@
         <v>50</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -2686,10 +2790,10 @@
         <v>102</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F24" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -2706,10 +2810,10 @@
         <v>34</v>
       </c>
       <c r="E25" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="F25" t="s">
         <v>142</v>
-      </c>
-      <c r="F25" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -2717,10 +2821,10 @@
         <v>115</v>
       </c>
       <c r="E26" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="F26" t="s">
         <v>144</v>
-      </c>
-      <c r="F26" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -2728,7 +2832,7 @@
         <v>66</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -2750,10 +2854,10 @@
         <v>105</v>
       </c>
       <c r="E29" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="F29" t="s">
         <v>146</v>
-      </c>
-      <c r="F29" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -2764,7 +2868,7 @@
         <v>65</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -2781,10 +2885,10 @@
         <v>45</v>
       </c>
       <c r="E31" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="F31" t="s">
         <v>148</v>
-      </c>
-      <c r="F31" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -2801,7 +2905,7 @@
         <v>76</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -2809,7 +2913,7 @@
         <v>67</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -2817,10 +2921,10 @@
         <v>68</v>
       </c>
       <c r="E34" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="F34" t="s">
         <v>150</v>
-      </c>
-      <c r="F34" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -2838,10 +2942,10 @@
         <v>71</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F37" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -2858,10 +2962,10 @@
         <v>58</v>
       </c>
       <c r="E38" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="F38" t="s">
         <v>153</v>
-      </c>
-      <c r="F38" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -2886,10 +2990,10 @@
         <v>44</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F40" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2906,10 +3010,10 @@
         <v>101</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F41" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -2926,19 +3030,23 @@
         <v>101</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F42" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup scale="21" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A753260-5018-4B3D-A2D6-F970E150F2D9}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:E81"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2953,13 +3061,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>122</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -2973,7 +3081,7 @@
         <v>23649844</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -2981,13 +3089,13 @@
         <v>9</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C3" s="2">
         <v>19001169</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -2995,13 +3103,13 @@
         <v>13</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C4" s="2">
         <v>16823806</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -3009,13 +3117,13 @@
         <v>13</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C5" s="2">
         <v>26053668</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -3029,7 +3137,7 @@
         <v>23649844</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -3037,13 +3145,13 @@
         <v>13</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C7" s="2">
         <v>18945794</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -3051,13 +3159,13 @@
         <v>13</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C8" s="2">
         <v>24128683</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -3065,7 +3173,7 @@
         <v>16</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C9" s="2">
         <v>26053668</v>
@@ -3083,7 +3191,7 @@
         <v>23649844</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -3091,13 +3199,13 @@
         <v>16</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C11" s="2">
         <v>30192380</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -3111,7 +3219,7 @@
         <v>23649844</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -3125,7 +3233,7 @@
         <v>23649844</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -3139,7 +3247,7 @@
         <v>23649844</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -3147,13 +3255,13 @@
         <v>19</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C15" s="8">
         <v>19151023</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -3161,13 +3269,13 @@
         <v>19</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C16" s="8">
         <v>24128683</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -3175,13 +3283,13 @@
         <v>19</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C17" s="8">
         <v>8042923</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -3189,13 +3297,13 @@
         <v>19</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C18" s="8">
         <v>6472420</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -3209,7 +3317,7 @@
         <v>23649844</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -3223,7 +3331,7 @@
         <v>23649844</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -3237,7 +3345,7 @@
         <v>23649844</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -3251,7 +3359,7 @@
         <v>23649844</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -3294,13 +3402,13 @@
         <v>43</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C28" s="2">
         <v>30842973</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -3315,13 +3423,13 @@
         <v>112</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C30" s="2">
         <v>39910058</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -3336,13 +3444,13 @@
         <v>45</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C32" s="8">
         <v>19961535</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -3350,13 +3458,13 @@
         <v>45</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C33" s="8">
         <v>9225322</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -3364,13 +3472,13 @@
         <v>45</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C34" s="8">
         <v>25701871</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -3378,13 +3486,13 @@
         <v>46</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C35" s="8">
         <v>24128683</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -3392,13 +3500,13 @@
         <v>46</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C36" s="8">
         <v>30842973</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -3412,7 +3520,7 @@
         <v>23649844</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -3420,13 +3528,13 @@
         <v>47</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C38" s="2">
         <v>39910058</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -3434,13 +3542,13 @@
         <v>114</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C39" s="2">
         <v>39910058</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -3448,13 +3556,13 @@
         <v>53</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C40" s="8">
         <v>30842973</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -3462,13 +3570,13 @@
         <v>53</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C41" s="8">
         <v>30697589</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -3482,7 +3590,7 @@
         <v>40343075</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -3490,13 +3598,13 @@
         <v>66</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C43" s="8">
         <v>16951681</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -3517,7 +3625,7 @@
         <v>23649844</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -3525,13 +3633,13 @@
         <v>57</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C46" s="8">
         <v>26896090</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -3545,7 +3653,7 @@
         <v>23649844</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -3553,13 +3661,13 @@
         <v>61</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C48" s="8">
         <v>21909802</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -3573,7 +3681,7 @@
         <v>23649844</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -3587,7 +3695,7 @@
         <v>23649844</v>
       </c>
       <c r="D50" s="11" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -3601,7 +3709,7 @@
         <v>23649844</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -3609,13 +3717,13 @@
         <v>68</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C52" s="8">
         <v>23261988</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -3637,13 +3745,13 @@
         <v>71</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C55" s="2">
         <v>23261988</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -3651,13 +3759,13 @@
         <v>72</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C56" s="8">
         <v>31695592</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -3672,13 +3780,13 @@
         <v>95</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C58" s="8">
         <v>30697589</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -3686,13 +3794,13 @@
         <v>96</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C59" s="8">
         <v>30697589</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -3700,13 +3808,13 @@
         <v>109</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C60" s="8">
         <v>30697589</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -3781,5 +3889,6 @@
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup scale="40" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>